<commit_message>
Continued progress on PDF fileds
</commit_message>
<xml_diff>
--- a/Pool Data Sheet Filler/Test Sheet.xlsx
+++ b/Pool Data Sheet Filler/Test Sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4537e0bdef8c4a1e/Documents/GitHub/Misc-Python-Stuff/Pool Data Sheet Filler/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="150" documentId="11_F25DC773A252ABDACC10489111DD68645ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C87179AC-A094-4DC7-9DBD-D773B60409BC}"/>
+  <xr:revisionPtr revIDLastSave="206" documentId="11_F25DC773A252ABDACC10489111DD68645ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78091C33-0414-4831-8FE2-BD93D6719D9E}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pool Data For Export" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
   <si>
     <t>Fraser</t>
   </si>
@@ -118,13 +118,52 @@
   </si>
   <si>
     <t>random@icould.com</t>
+  </si>
+  <si>
+    <t>General Information</t>
+  </si>
+  <si>
+    <t>Name of Pool:</t>
+  </si>
+  <si>
+    <t>Civic Address:</t>
+  </si>
+  <si>
+    <t>Pool Type:</t>
+  </si>
+  <si>
+    <t>Pool Type</t>
+  </si>
+  <si>
+    <t>Indoor/Outdoor</t>
+  </si>
+  <si>
+    <t>Public Pool</t>
+  </si>
+  <si>
+    <t>Commercial Pool</t>
+  </si>
+  <si>
+    <t>Hot Tub</t>
+  </si>
+  <si>
+    <t>Spray Pool</t>
+  </si>
+  <si>
+    <t>Wading Pool</t>
+  </si>
+  <si>
+    <t>Indoor</t>
+  </si>
+  <si>
+    <t>Outdoor</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -162,16 +201,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -201,6 +232,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -217,7 +254,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -225,23 +262,23 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="4"/>
-    <xf numFmtId="14" fontId="3" fillId="5" borderId="0" xfId="4" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="4" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="5" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="5"/>
+    <xf numFmtId="14" fontId="3" fillId="6" borderId="0" xfId="5" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="20% - Accent5" xfId="2" builtinId="46"/>
     <cellStyle name="20% - Accent6" xfId="3" builtinId="50"/>
+    <cellStyle name="40% - Accent5" xfId="5" builtinId="47"/>
     <cellStyle name="40% - Accent6" xfId="4" builtinId="51"/>
     <cellStyle name="Accent6" xfId="1" builtinId="49"/>
-    <cellStyle name="Hyperlink" xfId="5" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -520,25 +557,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="49" customWidth="1"/>
-    <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -546,132 +583,166 @@
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="8">
         <f ca="1">TODAY()</f>
-        <v>45916</v>
-      </c>
-      <c r="E3" s="4"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+        <v>45917</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="7" t="s">
         <v>20</v>
       </c>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>21</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="2"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>18</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>23</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="7" t="s">
         <v>24</v>
       </c>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>25</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="2"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="2" t="str">
+        <f>B3</f>
+        <v>AME test pool</v>
+      </c>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="4" t="str">
+        <f>B4</f>
+        <v>1175 Douglas St #912, Victoria, BC V8W 2E1</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>38</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A9:E9"/>
+  <mergeCells count="4">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A14:D14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D8" r:id="rId1" xr:uid="{9A463325-EB8C-4024-9F3F-B2342E38C117}"/>
@@ -681,12 +752,24 @@
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DBDA0B2E-73C7-461D-9A78-8C9C0FC3C8EE}">
           <x14:formula1>
             <xm:f>Backend!$A$2:$A$6</xm:f>
           </x14:formula1>
           <xm:sqref>B2</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7B628694-0BAE-40DE-9EB6-6794FE42A36A}">
+          <x14:formula1>
+            <xm:f>Backend!$B$2:$B$6</xm:f>
+          </x14:formula1>
+          <xm:sqref>B17</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{401B17CD-BB80-40BD-8320-79D75DC7CF0F}">
+          <x14:formula1>
+            <xm:f>Backend!$C$2:$C$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>D17</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -696,40 +779,69 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC180A74-45BA-42EE-9251-9C730233F3C6}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Intermediate changes, program doesn't work currently.
</commit_message>
<xml_diff>
--- a/Pool Data Sheet Filler/Test Sheet.xlsx
+++ b/Pool Data Sheet Filler/Test Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4537e0bdef8c4a1e/Documents/GitHub/Misc-Python-Stuff/Pool Data Sheet Filler/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="206" documentId="11_F25DC773A252ABDACC10489111DD68645ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78091C33-0414-4831-8FE2-BD93D6719D9E}"/>
+  <xr:revisionPtr revIDLastSave="283" documentId="11_F25DC773A252ABDACC10489111DD68645ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8109CF4B-794A-46EF-9CB4-34075F1E4F24}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
   <si>
     <t>Fraser</t>
   </si>
@@ -157,6 +157,18 @@
   </si>
   <si>
     <t>Outdoor</t>
+  </si>
+  <si>
+    <t>Text</t>
+  </si>
+  <si>
+    <t>Input Type</t>
+  </si>
+  <si>
+    <t>Checkbox</t>
+  </si>
+  <si>
+    <t>Health Authority</t>
   </si>
 </sst>
 </file>
@@ -265,12 +277,14 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="4" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="5"/>
-    <xf numFmtId="14" fontId="3" fillId="6" borderId="0" xfId="5" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="6" borderId="0" xfId="5" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -557,196 +571,181 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A2:B21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49" customWidth="1"/>
-    <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="63.5703125" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="B2" s="9"/>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="6" t="s">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="8">
+      <c r="B6" s="10">
         <f ca="1">TODAY()</f>
-        <v>45917</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+        <v>45918</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="B7" s="8"/>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B10" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="2" t="s">
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="B11" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="B12" s="9"/>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B14" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B15" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="2" t="s">
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="B16" s="7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="B17" s="9"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="2" t="str">
-        <f>B3</f>
+      <c r="B18" s="2" t="str">
+        <f>B4</f>
         <v>AME test pool</v>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="4" t="str">
-        <f>B4</f>
+      <c r="B19" s="4" t="str">
+        <f>B5</f>
         <v>1175 Douglas St #912, Victoria, BC V8W 2E1</v>
       </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B20" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="2" t="s">
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="B21" s="7" t="s">
         <v>38</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A17:B17"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="D8" r:id="rId1" xr:uid="{9A463325-EB8C-4024-9F3F-B2342E38C117}"/>
-    <hyperlink ref="D12" r:id="rId2" xr:uid="{F23C4D8F-D3A5-41F8-8768-957B6ED66387}"/>
+    <hyperlink ref="B16" r:id="rId1" xr:uid="{F23C4D8F-D3A5-41F8-8768-957B6ED66387}"/>
+    <hyperlink ref="B11" r:id="rId2" xr:uid="{9A463325-EB8C-4024-9F3F-B2342E38C117}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId3"/>
@@ -757,19 +756,19 @@
           <x14:formula1>
             <xm:f>Backend!$A$2:$A$6</xm:f>
           </x14:formula1>
-          <xm:sqref>B2</xm:sqref>
+          <xm:sqref>B3</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7B628694-0BAE-40DE-9EB6-6794FE42A36A}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E16A27BC-15E6-475F-BB89-94A0C07741A8}">
           <x14:formula1>
             <xm:f>Backend!$B$2:$B$6</xm:f>
           </x14:formula1>
-          <xm:sqref>B17</xm:sqref>
+          <xm:sqref>B20</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{401B17CD-BB80-40BD-8320-79D75DC7CF0F}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B3132453-0252-43A7-BEC0-13862065EF0E}">
           <x14:formula1>
             <xm:f>Backend!$C$2:$C$3</xm:f>
           </x14:formula1>
-          <xm:sqref>D17</xm:sqref>
+          <xm:sqref>B21</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -779,15 +778,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC180A74-45BA-42EE-9251-9C730233F3C6}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -797,8 +797,12 @@
       <c r="C1" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -808,8 +812,11 @@
       <c r="C2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -819,16 +826,22 @@
       <c r="C3" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -836,7 +849,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
A lot of error checking
</commit_message>
<xml_diff>
--- a/Pool Data Sheet Filler/Test Sheet.xlsx
+++ b/Pool Data Sheet Filler/Test Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4537e0bdef8c4a1e/Documents/GitHub/Misc-Python-Stuff/Pool Data Sheet Filler/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="283" documentId="11_F25DC773A252ABDACC10489111DD68645ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8109CF4B-794A-46EF-9CB4-34075F1E4F24}"/>
+  <xr:revisionPtr revIDLastSave="323" documentId="11_F25DC773A252ABDACC10489111DD68645ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32DB8DD1-56B5-476C-88EE-C044C9FA42D2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -277,14 +277,14 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="4" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="5"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="14" fontId="3" fillId="6" borderId="0" xfId="5" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="6" borderId="0" xfId="5" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -615,16 +615,16 @@
       <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="8">
         <f ca="1">TODAY()</f>
         <v>45918</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="8"/>
+      <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
@@ -752,12 +752,6 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DBDA0B2E-73C7-461D-9A78-8C9C0FC3C8EE}">
-          <x14:formula1>
-            <xm:f>Backend!$A$2:$A$6</xm:f>
-          </x14:formula1>
-          <xm:sqref>B3</xm:sqref>
-        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E16A27BC-15E6-475F-BB89-94A0C07741A8}">
           <x14:formula1>
             <xm:f>Backend!$B$2:$B$6</xm:f>
@@ -769,6 +763,12 @@
             <xm:f>Backend!$C$2:$C$3</xm:f>
           </x14:formula1>
           <xm:sqref>B21</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DBDA0B2E-73C7-461D-9A78-8C9C0FC3C8EE}">
+          <x14:formula1>
+            <xm:f>Backend!$A$2:$A$6</xm:f>
+          </x14:formula1>
+          <xm:sqref>B3</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -804,7 +804,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
@@ -818,7 +818,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B3" t="s">
         <v>34</v>
@@ -832,7 +832,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" t="s">
         <v>35</v>
@@ -843,7 +843,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" t="s">
         <v>36</v>
@@ -851,7 +851,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B6" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Progress on code, still doesn't work
</commit_message>
<xml_diff>
--- a/Pool Data Sheet Filler/Test Sheet.xlsx
+++ b/Pool Data Sheet Filler/Test Sheet.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4537e0bdef8c4a1e/Documents/GitHub/Misc-Python-Stuff/Pool Data Sheet Filler/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benne\GitHub\Misc-Python-Stuff\Pool Data Sheet Filler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="323" documentId="11_F25DC773A252ABDACC10489111DD68645ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32DB8DD1-56B5-476C-88EE-C044C9FA42D2}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D4BEAF-D5A2-4D72-895F-2C964EB7DD4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pool Data For Export" sheetId="1" r:id="rId1"/>
@@ -571,181 +571,182 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:B21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.5703125" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="63.5546875" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="9"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="B1" s="9"/>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B3" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B5" s="8">
         <f ca="1">TODAY()</f>
-        <v>45918</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+        <v>45924</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="10"/>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="B6" s="10"/>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B7" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B8" s="7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B9" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B10" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="9"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="B11" s="9"/>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B12" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B13" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B14" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B15" s="7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="9"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+      <c r="B16" s="9"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="2" t="str">
+      <c r="B17" s="2" t="str">
+        <f>B3</f>
+        <v>AME test pool</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="4" t="str">
         <f>B4</f>
-        <v>AME test pool</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B19" s="4" t="str">
-        <f>B5</f>
         <v>1175 Douglas St #912, Victoria, BC V8W 2E1</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B19" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B20" s="7" t="s">
         <v>38</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A16:B16"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B16" r:id="rId1" xr:uid="{F23C4D8F-D3A5-41F8-8768-957B6ED66387}"/>
-    <hyperlink ref="B11" r:id="rId2" xr:uid="{9A463325-EB8C-4024-9F3F-B2342E38C117}"/>
+    <hyperlink ref="B15" r:id="rId1" xr:uid="{F23C4D8F-D3A5-41F8-8768-957B6ED66387}"/>
+    <hyperlink ref="B10" r:id="rId2" xr:uid="{9A463325-EB8C-4024-9F3F-B2342E38C117}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId3"/>
@@ -756,19 +757,19 @@
           <x14:formula1>
             <xm:f>Backend!$B$2:$B$6</xm:f>
           </x14:formula1>
-          <xm:sqref>B20</xm:sqref>
+          <xm:sqref>B19</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B3132453-0252-43A7-BEC0-13862065EF0E}">
           <x14:formula1>
             <xm:f>Backend!$C$2:$C$3</xm:f>
           </x14:formula1>
-          <xm:sqref>B21</xm:sqref>
+          <xm:sqref>B20</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DBDA0B2E-73C7-461D-9A78-8C9C0FC3C8EE}">
           <x14:formula1>
             <xm:f>Backend!$A$2:$A$6</xm:f>
           </x14:formula1>
-          <xm:sqref>B3</xm:sqref>
+          <xm:sqref>B2</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -778,16 +779,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC180A74-45BA-42EE-9251-9C730233F3C6}">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -802,7 +804,7 @@
       </c>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -816,7 +818,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -830,7 +832,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -841,7 +843,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -849,7 +851,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Continued Adding Fields to JSON
</commit_message>
<xml_diff>
--- a/Pool Data Sheet Filler/Test Sheet.xlsx
+++ b/Pool Data Sheet Filler/Test Sheet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benne\GitHub\Misc-Python-Stuff\Pool Data Sheet Filler\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4537e0bdef8c4a1e/Documents/GitHub/Misc-Python-Stuff/Pool Data Sheet Filler/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D4BEAF-D5A2-4D72-895F-2C964EB7DD4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="176" documentId="13_ncr:1_{E2D4BEAF-D5A2-4D72-895F-2C964EB7DD4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E59A62FD-CD65-46BE-BFCC-B7FAF6105445}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pool Data For Export" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="83">
   <si>
     <t>Fraser</t>
   </si>
@@ -63,9 +63,6 @@
     <t>Application To:</t>
   </si>
   <si>
-    <t>Health Authority:</t>
-  </si>
-  <si>
     <t>Name of Pool</t>
   </si>
   <si>
@@ -78,9 +75,6 @@
     <t>Street Adress</t>
   </si>
   <si>
-    <t>Contact Information: Owner or Agent (Left blank in most cases, filled by owner)</t>
-  </si>
-  <si>
     <t>AME test pool</t>
   </si>
   <si>
@@ -93,21 +87,6 @@
     <t>Email</t>
   </si>
   <si>
-    <t>Contact Information: Person Applying for Construction Permit (if different from Owner)</t>
-  </si>
-  <si>
-    <t>John Q Public</t>
-  </si>
-  <si>
-    <t>721 Johnson Street, Victoria, BC, V8W 1M8</t>
-  </si>
-  <si>
-    <t>123-456-7890</t>
-  </si>
-  <si>
-    <t>random@gmail.com</t>
-  </si>
-  <si>
     <t>John Doe</t>
   </si>
   <si>
@@ -169,13 +148,151 @@
   </si>
   <si>
     <t>Health Authority</t>
+  </si>
+  <si>
+    <t>Owner's Confirmation of Commitment</t>
+  </si>
+  <si>
+    <t>Owner Name</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Contact Information: Owner or Agent</t>
+  </si>
+  <si>
+    <t>Contact Information: Person Applying for Construction Permit</t>
+  </si>
+  <si>
+    <t>Normally Filled out by owner, can be left blank</t>
+  </si>
+  <si>
+    <t>Owner Information</t>
+  </si>
+  <si>
+    <t>Designer Information (Append additional information for multiple designers)</t>
+  </si>
+  <si>
+    <t>Company (Legal Corporate)</t>
+  </si>
+  <si>
+    <t>The AME Consulting Group</t>
+  </si>
+  <si>
+    <t>Professional Designation</t>
+  </si>
+  <si>
+    <t>Arch</t>
+  </si>
+  <si>
+    <t>PEng</t>
+  </si>
+  <si>
+    <t>General Pool Parameters</t>
+  </si>
+  <si>
+    <t>Pool Volume: (m^3)</t>
+  </si>
+  <si>
+    <t>Turnover: (hours)</t>
+  </si>
+  <si>
+    <t>Design Re-circulation Flow Rate: (L/sec)</t>
+  </si>
+  <si>
+    <t>Pool Area (m^2)</t>
+  </si>
+  <si>
+    <t>Deck Area (m^2)</t>
+  </si>
+  <si>
+    <t>Minimum Water Depth</t>
+  </si>
+  <si>
+    <t>Maximum Water Depth</t>
+  </si>
+  <si>
+    <t>Shallow Bathing Load</t>
+  </si>
+  <si>
+    <t>Deep Bathing Load</t>
+  </si>
+  <si>
+    <t>Total Bathing Load</t>
+  </si>
+  <si>
+    <t>Pool Basin Color</t>
+  </si>
+  <si>
+    <t>Complies with Pool Regulations</t>
+  </si>
+  <si>
+    <t>Yes/No</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Filters</t>
+  </si>
+  <si>
+    <t>Modify Cell to exclude ramps</t>
+  </si>
+  <si>
+    <t>Sand</t>
+  </si>
+  <si>
+    <t>Pressure</t>
+  </si>
+  <si>
+    <t>Vacuum</t>
+  </si>
+  <si>
+    <t>Gravity</t>
+  </si>
+  <si>
+    <t>NSF Approved</t>
+  </si>
+  <si>
+    <t>Pressure Gauge Quantity</t>
+  </si>
+  <si>
+    <t>Vacuum Gauge Quantity</t>
+  </si>
+  <si>
+    <t>Temperature Gauge Quantity</t>
+  </si>
+  <si>
+    <t>Disinfection</t>
+  </si>
+  <si>
+    <t>Hypochlorite</t>
+  </si>
+  <si>
+    <t>Chlorine Gas</t>
+  </si>
+  <si>
+    <t>Stabilized Chlorine</t>
+  </si>
+  <si>
+    <t>Bromine</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Blue</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -213,8 +330,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -250,8 +373,19 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -259,16 +393,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="6">
+  <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3"/>
@@ -280,20 +446,37 @@
     <xf numFmtId="14" fontId="3" fillId="6" borderId="0" xfId="5" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="7"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="3" applyBorder="1"/>
+    <xf numFmtId="14" fontId="3" fillId="5" borderId="1" xfId="4" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="5" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="4" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="8">
     <cellStyle name="20% - Accent5" xfId="2" builtinId="46"/>
     <cellStyle name="20% - Accent6" xfId="3" builtinId="50"/>
     <cellStyle name="40% - Accent5" xfId="5" builtinId="47"/>
     <cellStyle name="40% - Accent6" xfId="4" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="7" builtinId="52"/>
     <cellStyle name="Accent6" xfId="1" builtinId="49"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Note" xfId="6" builtinId="10"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -572,204 +755,536 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.5546875" customWidth="1"/>
-    <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="63.5703125" customWidth="1"/>
+    <col min="3" max="3" width="63.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="9"/>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B1" s="13"/>
+      <c r="C1" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>9</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
-        <v>10</v>
       </c>
       <c r="B5" s="8">
         <f ca="1">TODAY()</f>
-        <v>45924</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="14"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="10"/>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="B8" s="7"/>
+      <c r="C8" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="13"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B12" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="7" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" s="13"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="7"/>
+      <c r="C17" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="11" t="str">
+        <f>B2</f>
+        <v>Fraser</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" s="12">
+        <f ca="1">B5</f>
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="13" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="3" t="s">
+      <c r="B20" s="13"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="9"/>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" s="9"/>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="2" t="str">
+      <c r="B21" s="2" t="str">
         <f>B3</f>
         <v>AME test pool</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B18" s="4" t="str">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="4" t="str">
         <f>B4</f>
         <v>1175 Douglas St #912, Victoria, BC V8W 2E1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" s="13"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" s="13"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B31" s="4" t="str">
+        <f>B12</f>
+        <v>John Doe</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B34" s="2" t="str">
+        <f>B13</f>
+        <v>638 Smithe St Suite 200, Vancouver, BC V6B 1E3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B35" s="4" t="str">
+        <f>B14</f>
+        <v>098-765-4321</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B36" s="2" t="str">
+        <f>B15</f>
+        <v>random@icould.com</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B37" s="13"/>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" s="15">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B39" s="16">
+        <v>2.33</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B40" s="15">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41" s="16">
         <v>30</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>38</v>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B42" s="15">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B43" s="16">
+        <v>1</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B44" s="15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B45" s="16">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B46" s="15">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B47" s="17">
+        <f>SUM(B45:B46)</f>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B48" s="15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B49" s="16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B50" s="15" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B51" s="16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B52" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B53" s="16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B54" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B55" s="16" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="8">
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A30:B30"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A20:B20"/>
     <mergeCell ref="A16:B16"/>
   </mergeCells>
+  <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="B15" r:id="rId1" xr:uid="{F23C4D8F-D3A5-41F8-8768-957B6ED66387}"/>
-    <hyperlink ref="B10" r:id="rId2" xr:uid="{9A463325-EB8C-4024-9F3F-B2342E38C117}"/>
+    <hyperlink ref="B29" r:id="rId2" xr:uid="{7C1EE75F-8A56-4E1F-8F6D-E3D927261E7F}"/>
+    <hyperlink ref="B35" r:id="rId3" display="random@icould.com" xr:uid="{0D1B7BBF-15B3-4CFC-9039-2B5392E32994}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="7">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E16A27BC-15E6-475F-BB89-94A0C07741A8}">
           <x14:formula1>
             <xm:f>Backend!$B$2:$B$6</xm:f>
           </x14:formula1>
-          <xm:sqref>B19</xm:sqref>
+          <xm:sqref>B23</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B3132453-0252-43A7-BEC0-13862065EF0E}">
           <x14:formula1>
             <xm:f>Backend!$C$2:$C$3</xm:f>
           </x14:formula1>
-          <xm:sqref>B20</xm:sqref>
+          <xm:sqref>B24</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DBDA0B2E-73C7-461D-9A78-8C9C0FC3C8EE}">
           <x14:formula1>
             <xm:f>Backend!$A$2:$A$6</xm:f>
           </x14:formula1>
           <xm:sqref>B2</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{30E8FBE2-C2FC-4B6D-9F98-1AD125B8C425}">
+          <x14:formula1>
+            <xm:f>Backend!$E$2:$E$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>B32</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D7F0EB7B-BBFF-45D3-B222-8DBEA2A4E2AA}">
+          <x14:formula1>
+            <xm:f>Backend!$F$2:$F$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>B49 B51</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{85EB1F5D-2C0D-4619-81F3-F49B63FA8937}">
+          <x14:formula1>
+            <xm:f>Backend!$G$2:$G$6</xm:f>
+          </x14:formula1>
+          <xm:sqref>B50</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3BF7E381-8828-457B-A727-E2C5CC93B0AF}">
+          <x14:formula1>
+            <xm:f>Backend!$H$2:$H$6</xm:f>
+          </x14:formula1>
+          <xm:sqref>B55</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -780,83 +1295,138 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC180A74-45BA-42EE-9251-9C730233F3C6}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s">
         <v>33</v>
       </c>
-      <c r="C2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G2" t="s">
+        <v>68</v>
+      </c>
+      <c r="H2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+      <c r="E3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" t="s">
+        <v>79</v>
+      </c>
+      <c r="H3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+      <c r="G4" t="s">
+        <v>69</v>
+      </c>
+      <c r="H4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="G5" t="s">
+        <v>70</v>
+      </c>
+      <c r="H5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>30</v>
+      </c>
+      <c r="G6" t="s">
+        <v>71</v>
+      </c>
+      <c r="H6" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
More fields added to PDF
</commit_message>
<xml_diff>
--- a/Pool Data Sheet Filler/Test Sheet.xlsx
+++ b/Pool Data Sheet Filler/Test Sheet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4537e0bdef8c4a1e/Documents/GitHub/Misc-Python-Stuff/Pool Data Sheet Filler/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benne\GitHub\Misc-Python-Stuff\Pool Data Sheet Filler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="176" documentId="13_ncr:1_{E2D4BEAF-D5A2-4D72-895F-2C964EB7DD4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E59A62FD-CD65-46BE-BFCC-B7FAF6105445}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4922D1BC-07C8-4760-BE39-F55E3BEB786D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pool Data For Export" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="84">
   <si>
     <t>Fraser</t>
   </si>
@@ -286,6 +286,9 @@
   </si>
   <si>
     <t>Blue</t>
+  </si>
+  <si>
+    <t>D.E.</t>
   </si>
 </sst>
 </file>
@@ -452,12 +455,6 @@
     <xf numFmtId="14" fontId="3" fillId="5" borderId="1" xfId="4" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -466,6 +463,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="4" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -756,25 +759,25 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:C55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="36.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.5703125" customWidth="1"/>
-    <col min="3" max="3" width="63.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="63.5546875" customWidth="1"/>
+    <col min="3" max="3" width="63.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="13"/>
+      <c r="B1" s="16"/>
       <c r="C1" s="9" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>36</v>
       </c>
@@ -782,7 +785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>8</v>
       </c>
@@ -790,7 +793,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>11</v>
       </c>
@@ -798,22 +801,22 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="8">
         <f ca="1">TODAY()</f>
-        <v>45928</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="14"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B6" s="17"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
@@ -822,7 +825,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>13</v>
       </c>
@@ -831,7 +834,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>14</v>
       </c>
@@ -840,7 +843,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>15</v>
       </c>
@@ -849,13 +852,13 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="13" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="13"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B11" s="16"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>6</v>
       </c>
@@ -863,7 +866,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>13</v>
       </c>
@@ -871,7 +874,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>14</v>
       </c>
@@ -879,7 +882,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>15</v>
       </c>
@@ -887,13 +890,13 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="B16" s="13"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B16" s="16"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>38</v>
       </c>
@@ -902,7 +905,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>36</v>
       </c>
@@ -911,22 +914,22 @@
         <v>Fraser</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B19" s="12">
         <f ca="1">B5</f>
-        <v>45928</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="13" t="s">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="13"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B20" s="16"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>21</v>
       </c>
@@ -935,7 +938,7 @@
         <v>AME test pool</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>22</v>
       </c>
@@ -944,15 +947,15 @@
         <v>1175 Douglas St #912, Victoria, BC V8W 2E1</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>25</v>
       </c>
@@ -960,13 +963,13 @@
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="13" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="B25" s="13"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B25" s="16"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>6</v>
       </c>
@@ -977,7 +980,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
         <v>13</v>
       </c>
@@ -988,7 +991,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>14</v>
       </c>
@@ -999,7 +1002,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
         <v>15</v>
       </c>
@@ -1010,13 +1013,13 @@
         <v>42</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="13" t="s">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="B30" s="13"/>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B30" s="16"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>6</v>
       </c>
@@ -1025,7 +1028,7 @@
         <v>John Doe</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>47</v>
       </c>
@@ -1033,7 +1036,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
         <v>45</v>
       </c>
@@ -1041,7 +1044,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>13</v>
       </c>
@@ -1050,7 +1053,7 @@
         <v>638 Smithe St Suite 200, Vancouver, BC V6B 1E3</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
         <v>14</v>
       </c>
@@ -1059,7 +1062,7 @@
         <v>098-765-4321</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>15</v>
       </c>
@@ -1068,157 +1071,157 @@
         <v>random@icould.com</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="13" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="B37" s="13"/>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B37" s="16"/>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B38" s="15">
+      <c r="B38" s="13">
         <v>300</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B39" s="16">
+      <c r="B39" s="14">
         <v>2.33</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B40" s="15">
+      <c r="B40" s="13">
         <v>1200</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B41" s="16">
+      <c r="B41" s="14">
         <v>30</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B42" s="15">
+      <c r="B42" s="13">
         <v>20</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B43" s="16">
+      <c r="B43" s="14">
         <v>1</v>
       </c>
       <c r="C43" s="10" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B44" s="15">
+      <c r="B44" s="13">
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B45" s="16">
+      <c r="B45" s="14">
         <v>100</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B46" s="15">
+      <c r="B46" s="13">
         <v>100</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B47" s="17">
+      <c r="B47" s="15">
         <f>SUM(B45:B46)</f>
         <v>200</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B48" s="15" t="s">
+      <c r="B48" s="13" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B49" s="16" t="s">
+      <c r="B49" s="14" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B50" s="15" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B50" s="13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B51" s="16" t="s">
+      <c r="B51" s="14" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="B52" s="15">
+      <c r="B52" s="13">
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B53" s="16">
+      <c r="B53" s="14">
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B54" s="15">
+      <c r="B54" s="13">
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="B55" s="16" t="s">
+      <c r="B55" s="14" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1296,17 +1299,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC180A74-45BA-42EE-9251-9C730233F3C6}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.109375" customWidth="1"/>
     <col min="8" max="8" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1332,7 +1336,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1358,7 +1362,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1378,13 +1382,13 @@
         <v>65</v>
       </c>
       <c r="G3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="H3" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -1401,7 +1405,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -1415,7 +1419,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Updated gitignore to ignore pycache
</commit_message>
<xml_diff>
--- a/Pool Data Sheet Filler/Test Sheet.xlsx
+++ b/Pool Data Sheet Filler/Test Sheet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benne\GitHub\Misc-Python-Stuff\Pool Data Sheet Filler\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4537e0bdef8c4a1e/Documents/GitHub/Misc-Python-Stuff/Pool Data Sheet Filler/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4922D1BC-07C8-4760-BE39-F55E3BEB786D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pool Data For Export" sheetId="1" r:id="rId1"/>
@@ -759,16 +759,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:C55"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.5546875" customWidth="1"/>
-    <col min="3" max="3" width="63.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="63.5703125" customWidth="1"/>
+    <col min="3" max="3" width="63.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
         <v>7</v>
       </c>
@@ -777,7 +777,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>36</v>
       </c>
@@ -785,7 +785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>8</v>
       </c>
@@ -793,7 +793,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>11</v>
       </c>
@@ -801,7 +801,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>9</v>
       </c>
@@ -810,13 +810,13 @@
         <v>45931</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
         <v>40</v>
       </c>
       <c r="B6" s="17"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
@@ -825,7 +825,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>13</v>
       </c>
@@ -834,7 +834,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>14</v>
       </c>
@@ -843,7 +843,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>15</v>
       </c>
@@ -852,13 +852,13 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
         <v>41</v>
       </c>
       <c r="B11" s="16"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>6</v>
       </c>
@@ -866,7 +866,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>13</v>
       </c>
@@ -874,7 +874,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>14</v>
       </c>
@@ -882,7 +882,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>15</v>
       </c>
@@ -890,13 +890,13 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
         <v>37</v>
       </c>
       <c r="B16" s="16"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>38</v>
       </c>
@@ -905,7 +905,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>36</v>
       </c>
@@ -914,7 +914,7 @@
         <v>Fraser</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>9</v>
       </c>
@@ -923,13 +923,13 @@
         <v>45931</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
         <v>20</v>
       </c>
       <c r="B20" s="16"/>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>21</v>
       </c>
@@ -938,7 +938,7 @@
         <v>AME test pool</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>22</v>
       </c>
@@ -947,7 +947,7 @@
         <v>1175 Douglas St #912, Victoria, BC V8W 2E1</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>23</v>
       </c>
@@ -955,7 +955,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>25</v>
       </c>
@@ -963,13 +963,13 @@
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="16" t="s">
         <v>43</v>
       </c>
       <c r="B25" s="16"/>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>6</v>
       </c>
@@ -980,7 +980,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>13</v>
       </c>
@@ -991,7 +991,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>14</v>
       </c>
@@ -1002,7 +1002,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>15</v>
       </c>
@@ -1013,13 +1013,13 @@
         <v>42</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="16" t="s">
         <v>44</v>
       </c>
       <c r="B30" s="16"/>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>6</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>John Doe</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>47</v>
       </c>
@@ -1036,7 +1036,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>45</v>
       </c>
@@ -1044,7 +1044,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>13</v>
       </c>
@@ -1053,7 +1053,7 @@
         <v>638 Smithe St Suite 200, Vancouver, BC V6B 1E3</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>14</v>
       </c>
@@ -1062,7 +1062,7 @@
         <v>098-765-4321</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>15</v>
       </c>
@@ -1071,13 +1071,13 @@
         <v>random@icould.com</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="16" t="s">
         <v>50</v>
       </c>
       <c r="B37" s="16"/>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>51</v>
       </c>
@@ -1085,7 +1085,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>52</v>
       </c>
@@ -1093,7 +1093,7 @@
         <v>2.33</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
         <v>53</v>
       </c>
@@ -1101,7 +1101,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>54</v>
       </c>
@@ -1109,7 +1109,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>55</v>
       </c>
@@ -1117,7 +1117,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>56</v>
       </c>
@@ -1128,7 +1128,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>57</v>
       </c>
@@ -1136,7 +1136,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>58</v>
       </c>
@@ -1144,7 +1144,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>59</v>
       </c>
@@ -1152,7 +1152,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>60</v>
       </c>
@@ -1161,7 +1161,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
         <v>61</v>
       </c>
@@ -1169,7 +1169,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>62</v>
       </c>
@@ -1177,7 +1177,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>66</v>
       </c>
@@ -1185,7 +1185,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>72</v>
       </c>
@@ -1193,7 +1193,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
         <v>73</v>
       </c>
@@ -1201,7 +1201,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>74</v>
       </c>
@@ -1209,7 +1209,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
         <v>75</v>
       </c>
@@ -1217,7 +1217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
         <v>76</v>
       </c>
@@ -1299,18 +1299,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC180A74-45BA-42EE-9251-9C730233F3C6}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.109375" customWidth="1"/>
+    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.140625" customWidth="1"/>
     <col min="8" max="8" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1336,7 +1336,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1362,7 +1362,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1388,7 +1388,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -1405,7 +1405,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -1419,7 +1419,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Added ability to update configuation file fields from excel sheet
</commit_message>
<xml_diff>
--- a/Pool Data Sheet Filler/Test Sheet.xlsx
+++ b/Pool Data Sheet Filler/Test Sheet.xlsx
@@ -5,19 +5,19 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4537e0bdef8c4a1e/Documents/GitHub/Misc-Python-Stuff/Pool Data Sheet Filler/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benne\GitHub\Misc-Python-Stuff\Pool Data Sheet Filler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="178" documentId="13_ncr:1_{911F8ABB-7C8C-4006-93F8-A150D2B68EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64F3D220-D794-4F71-9AA1-3756E0EE02F0}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21DAD4A1-FDED-4752-BA45-127BD1670C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pool Data For Export" sheetId="1" r:id="rId1"/>
     <sheet name="Backend" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pool Data For Export'!$I$80:$J$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pool Data For Export'!$K$82:$L$82</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="128">
   <si>
     <t>Fraser</t>
   </si>
@@ -434,6 +434,18 @@
   </si>
   <si>
     <t>points</t>
+  </si>
+  <si>
+    <t>Override name</t>
+  </si>
+  <si>
+    <t>Override value</t>
+  </si>
+  <si>
+    <t>text x offset</t>
+  </si>
+  <si>
+    <t>text y offset</t>
   </si>
 </sst>
 </file>
@@ -582,7 +594,7 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3"/>
@@ -609,17 +621,11 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="4" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -638,14 +644,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Note" xfId="6" builtinId="10"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill>
@@ -691,14 +690,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
+          <bgColor theme="7" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -979,21 +978,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K118"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:M120"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="150.28515625" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" customWidth="1"/>
-    <col min="3" max="3" width="58.5703125" customWidth="1"/>
-    <col min="4" max="8" width="21.28515625" customWidth="1"/>
-    <col min="9" max="9" width="54.7109375" customWidth="1"/>
-    <col min="10" max="10" width="63.5703125" customWidth="1"/>
-    <col min="11" max="11" width="63.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.85546875" customWidth="1"/>
-    <col min="13" max="15" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="91.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" customWidth="1"/>
+    <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="54.6640625" customWidth="1"/>
+    <col min="12" max="12" width="63.5546875" customWidth="1"/>
+    <col min="13" max="13" width="63.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.88671875" customWidth="1"/>
+    <col min="15" max="17" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>120</v>
       </c>
@@ -1018,17 +1022,23 @@
       <c r="H1" t="s">
         <v>122</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" t="s">
+        <v>124</v>
+      </c>
+      <c r="J1" t="s">
+        <v>125</v>
+      </c>
+      <c r="K1" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="20"/>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="18"/>
+      <c r="M1" s="9" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="str">
-        <f>_xlfn.CONCAT($I$1," ",I2)</f>
+        <f>_xlfn.CONCAT($K$1," ",K2)</f>
         <v>Application To: Health Authority</v>
       </c>
       <c r="B2" t="s">
@@ -1044,8 +1054,8 @@
         <v>158</v>
       </c>
       <c r="F2" t="str" cm="1">
-        <f t="array" aca="1" ref="F2" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J2),"$"))</f>
-        <v>J2</v>
+        <f t="array" aca="1" ref="F2" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L2),"$"))</f>
+        <v>L2</v>
       </c>
       <c r="G2">
         <v>2</v>
@@ -1053,78 +1063,82 @@
       <c r="H2" t="s">
         <v>123</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="K2" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>257</v>
+        <v>41</v>
       </c>
       <c r="E3">
         <v>158</v>
       </c>
-      <c r="I3" s="5"/>
-      <c r="J3" s="3"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K3" s="5"/>
+      <c r="L3" s="3"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>1</v>
       </c>
       <c r="D4">
-        <v>257</v>
+        <v>162</v>
       </c>
       <c r="E4">
         <v>158</v>
       </c>
-      <c r="I4" s="5"/>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K4" s="5"/>
+      <c r="L4" s="3"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>2</v>
       </c>
       <c r="D5">
-        <v>257</v>
+        <v>369</v>
       </c>
       <c r="E5">
         <v>158</v>
       </c>
-      <c r="I5" s="5"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K5" s="5"/>
+      <c r="L5" s="3"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
         <v>3</v>
       </c>
       <c r="D6">
-        <v>257</v>
+        <v>482</v>
       </c>
       <c r="E6">
         <v>158</v>
       </c>
-      <c r="I6" s="5"/>
-      <c r="J6" s="3"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K6" s="5"/>
+      <c r="L6" s="3"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="str">
-        <f t="shared" ref="A7:A9" si="0">_xlfn.CONCAT($I$1," ",I7)</f>
+        <f t="shared" ref="A7:A9" si="0">_xlfn.CONCAT($K$1," ",K7)</f>
         <v>Application To: Name of Pool</v>
       </c>
       <c r="B7" t="s">
         <v>78</v>
       </c>
-      <c r="D7" s="16"/>
-      <c r="E7" s="19"/>
+      <c r="D7">
+        <v>31</v>
+      </c>
+      <c r="E7">
+        <v>216</v>
+      </c>
       <c r="F7" t="str" cm="1">
-        <f t="array" aca="1" ref="F7" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J7),"$"))</f>
-        <v>J7</v>
+        <f t="array" aca="1" ref="F7" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L7),"$"))</f>
+        <v>L7</v>
       </c>
       <c r="G7">
         <v>2</v>
@@ -1132,14 +1146,14 @@
       <c r="H7" t="s">
         <v>123</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="K7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J7" s="7" t="s">
+      <c r="L7" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" t="str">
         <f t="shared" si="0"/>
         <v>Application To: Street Adress</v>
@@ -1147,9 +1161,15 @@
       <c r="B8" t="s">
         <v>78</v>
       </c>
+      <c r="D8">
+        <v>31</v>
+      </c>
+      <c r="E8">
+        <v>245</v>
+      </c>
       <c r="F8" t="str" cm="1">
-        <f t="array" aca="1" ref="F8" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J8),"$"))</f>
-        <v>J8</v>
+        <f t="array" aca="1" ref="F8" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L8),"$"))</f>
+        <v>L8</v>
       </c>
       <c r="G8">
         <v>2</v>
@@ -1157,14 +1177,14 @@
       <c r="H8" t="s">
         <v>123</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="K8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="L8" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="str">
         <f t="shared" si="0"/>
         <v>Application To: Date</v>
@@ -1172,9 +1192,15 @@
       <c r="B9" t="s">
         <v>78</v>
       </c>
+      <c r="D9">
+        <v>405</v>
+      </c>
+      <c r="E9">
+        <v>216</v>
+      </c>
       <c r="F9" t="str" cm="1">
-        <f t="array" aca="1" ref="F9" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J9),"$"))</f>
-        <v>J9</v>
+        <f t="array" aca="1" ref="F9" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L9),"$"))</f>
+        <v>L9</v>
       </c>
       <c r="G9">
         <v>2</v>
@@ -1182,31 +1208,37 @@
       <c r="H9" t="s">
         <v>123</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="K9" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J9" s="8">
+      <c r="L9" s="8">
         <f ca="1">TODAY()</f>
-        <v>45949</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I10" s="21" t="s">
+        <v>45957</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="K10" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="J10" s="21"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L10" s="19"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" t="str">
-        <f>_xlfn.CONCAT($I$10," ",I11)</f>
+        <f>_xlfn.CONCAT($K$10," ",K11)</f>
         <v>Contact Information: Owner or Agent Name</v>
       </c>
       <c r="B11" t="s">
         <v>78</v>
       </c>
+      <c r="D11">
+        <v>31</v>
+      </c>
+      <c r="E11">
+        <v>295</v>
+      </c>
       <c r="F11" t="str" cm="1">
-        <f t="array" aca="1" ref="F11" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J11),"$"))</f>
-        <v>J11</v>
+        <f t="array" aca="1" ref="F11" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L11),"$"))</f>
+        <v>L11</v>
       </c>
       <c r="G11">
         <v>2</v>
@@ -1214,25 +1246,31 @@
       <c r="H11" t="s">
         <v>123</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="K11" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="J11" s="3"/>
-      <c r="K11" s="10" t="s">
+      <c r="L11" s="3"/>
+      <c r="M11" s="10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" t="str">
-        <f t="shared" ref="A12:A14" si="1">_xlfn.CONCAT($I$10," ",I12)</f>
+        <f t="shared" ref="A12:A14" si="1">_xlfn.CONCAT($K$10," ",K12)</f>
         <v>Contact Information: Owner or Agent Address</v>
       </c>
       <c r="B12" t="s">
         <v>78</v>
       </c>
+      <c r="D12">
+        <v>31</v>
+      </c>
+      <c r="E12">
+        <v>322</v>
+      </c>
       <c r="F12" t="str" cm="1">
-        <f t="array" aca="1" ref="F12" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J12),"$"))</f>
-        <v>J12</v>
+        <f t="array" aca="1" ref="F12" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L12),"$"))</f>
+        <v>L12</v>
       </c>
       <c r="G12">
         <v>2</v>
@@ -1240,15 +1278,15 @@
       <c r="H12" t="s">
         <v>123</v>
       </c>
-      <c r="I12" s="6" t="s">
+      <c r="K12" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="J12" s="7"/>
-      <c r="K12" s="10" t="s">
+      <c r="L12" s="7"/>
+      <c r="M12" s="10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" t="str">
         <f t="shared" si="1"/>
         <v>Contact Information: Owner or Agent Phone Number</v>
@@ -1256,9 +1294,15 @@
       <c r="B13" t="s">
         <v>78</v>
       </c>
+      <c r="D13">
+        <v>31</v>
+      </c>
+      <c r="E13">
+        <v>351</v>
+      </c>
       <c r="F13" t="str" cm="1">
-        <f t="array" aca="1" ref="F13" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J13),"$"))</f>
-        <v>J13</v>
+        <f t="array" aca="1" ref="F13" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L13),"$"))</f>
+        <v>L13</v>
       </c>
       <c r="G13">
         <v>2</v>
@@ -1266,15 +1310,15 @@
       <c r="H13" t="s">
         <v>123</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="K13" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="J13" s="3"/>
-      <c r="K13" s="10" t="s">
+      <c r="L13" s="3"/>
+      <c r="M13" s="10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" t="str">
         <f t="shared" si="1"/>
         <v>Contact Information: Owner or Agent Email</v>
@@ -1282,9 +1326,15 @@
       <c r="B14" t="s">
         <v>78</v>
       </c>
+      <c r="D14">
+        <v>249</v>
+      </c>
+      <c r="E14">
+        <v>351</v>
+      </c>
       <c r="F14" t="str" cm="1">
-        <f t="array" aca="1" ref="F14" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J14),"$"))</f>
-        <v>J14</v>
+        <f t="array" aca="1" ref="F14" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L14),"$"))</f>
+        <v>L14</v>
       </c>
       <c r="G14">
         <v>2</v>
@@ -1292,38 +1342,40 @@
       <c r="H14" t="s">
         <v>123</v>
       </c>
-      <c r="I14" s="6" t="s">
+      <c r="K14" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="J14" s="7" t="str">
-        <f>K14</f>
+      <c r="L14" s="7" t="str">
+        <f>M14</f>
         <v>Normally Filled out by owner, can be left blank</v>
       </c>
-      <c r="K14" s="10" t="s">
+      <c r="M14" s="10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I15" s="20" t="s">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="K15" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="J15" s="20"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L15" s="18"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" t="str">
-        <f>_xlfn.CONCAT($I$15," ",I16)</f>
+        <f>_xlfn.CONCAT($K$15," ",K16)</f>
         <v>Contact Information: Person Applying for Construction Permit Name</v>
       </c>
       <c r="B16" t="s">
         <v>78</v>
       </c>
-      <c r="D16" t="str" cm="1">
-        <f t="array" aca="1" ref="D16" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J2),"$"))</f>
-        <v>J2</v>
+      <c r="D16">
+        <v>31</v>
+      </c>
+      <c r="E16">
+        <v>402</v>
       </c>
       <c r="F16" t="str" cm="1">
-        <f t="array" aca="1" ref="F16" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J16),"$"))</f>
-        <v>J16</v>
+        <f t="array" aca="1" ref="F16" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L16),"$"))</f>
+        <v>L16</v>
       </c>
       <c r="G16">
         <v>2</v>
@@ -1331,24 +1383,30 @@
       <c r="H16" t="s">
         <v>123</v>
       </c>
-      <c r="I16" s="5" t="s">
+      <c r="K16" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="J16" s="3" t="s">
+      <c r="L16" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" t="str">
-        <f t="shared" ref="A17:A19" si="2">_xlfn.CONCAT($I$15," ",I17)</f>
+        <f t="shared" ref="A17:A19" si="2">_xlfn.CONCAT($K$15," ",K17)</f>
         <v>Contact Information: Person Applying for Construction Permit Address</v>
       </c>
       <c r="B17" t="s">
         <v>78</v>
       </c>
+      <c r="D17">
+        <v>31</v>
+      </c>
+      <c r="E17">
+        <v>429</v>
+      </c>
       <c r="F17" t="str" cm="1">
-        <f t="array" aca="1" ref="F17" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J17),"$"))</f>
-        <v>J17</v>
+        <f t="array" aca="1" ref="F17" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L17),"$"))</f>
+        <v>L17</v>
       </c>
       <c r="G17">
         <v>2</v>
@@ -1356,14 +1414,14 @@
       <c r="H17" t="s">
         <v>123</v>
       </c>
-      <c r="I17" s="6" t="s">
+      <c r="K17" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="J17" s="7" t="s">
+      <c r="L17" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" t="str">
         <f t="shared" si="2"/>
         <v>Contact Information: Person Applying for Construction Permit Phone Number</v>
@@ -1371,9 +1429,15 @@
       <c r="B18" t="s">
         <v>78</v>
       </c>
+      <c r="D18">
+        <v>31</v>
+      </c>
+      <c r="E18">
+        <v>458</v>
+      </c>
       <c r="F18" t="str" cm="1">
-        <f t="array" aca="1" ref="F18" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J18),"$"))</f>
-        <v>J18</v>
+        <f t="array" aca="1" ref="F18" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L18),"$"))</f>
+        <v>L18</v>
       </c>
       <c r="G18">
         <v>2</v>
@@ -1381,14 +1445,14 @@
       <c r="H18" t="s">
         <v>123</v>
       </c>
-      <c r="I18" s="5" t="s">
+      <c r="K18" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="J18" s="3" t="s">
+      <c r="L18" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="str">
         <f t="shared" si="2"/>
         <v>Contact Information: Person Applying for Construction Permit Email</v>
@@ -1396,9 +1460,15 @@
       <c r="B19" t="s">
         <v>78</v>
       </c>
+      <c r="D19">
+        <v>249</v>
+      </c>
+      <c r="E19">
+        <v>458</v>
+      </c>
       <c r="F19" t="str" cm="1">
-        <f t="array" aca="1" ref="F19" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J19),"$"))</f>
-        <v>J19</v>
+        <f t="array" aca="1" ref="F19" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L19),"$"))</f>
+        <v>L19</v>
       </c>
       <c r="G19">
         <v>2</v>
@@ -1406,30 +1476,36 @@
       <c r="H19" t="s">
         <v>123</v>
       </c>
-      <c r="I19" s="6" t="s">
+      <c r="K19" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="J19" s="7" t="s">
+      <c r="L19" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I20" s="20" t="s">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="K20" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="J20" s="20"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L20" s="18"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" t="str">
-        <f>_xlfn.CONCAT($I$20,": ",I21)</f>
+        <f>_xlfn.CONCAT($K$20,": ",K21)</f>
         <v>Owner's Confirmation of Commitment: Owner Name</v>
       </c>
       <c r="B21" t="s">
         <v>78</v>
       </c>
+      <c r="D21">
+        <v>46</v>
+      </c>
+      <c r="E21">
+        <v>493</v>
+      </c>
       <c r="F21" t="str" cm="1">
-        <f t="array" aca="1" ref="F21" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J21),"$"))</f>
-        <v>J21</v>
+        <f t="array" aca="1" ref="F21" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L21),"$"))</f>
+        <v>L21</v>
       </c>
       <c r="G21">
         <v>2</v>
@@ -1437,350 +1513,469 @@
       <c r="H21" t="s">
         <v>123</v>
       </c>
-      <c r="I21" s="6" t="s">
+      <c r="I21" t="s">
+        <v>126</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="J21" s="7"/>
-      <c r="K21" s="10" t="s">
+      <c r="L21" s="7"/>
+      <c r="M21" s="10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" t="str">
-        <f t="shared" ref="A22:A23" si="3">_xlfn.CONCAT($I$20,": ",I22)</f>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I22" t="s">
+        <v>127</v>
+      </c>
+      <c r="J22">
+        <v>2</v>
+      </c>
+      <c r="K22" s="6"/>
+      <c r="L22" s="7"/>
+      <c r="M22" s="10"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A23" t="str">
+        <f t="shared" ref="A23:A25" si="3">_xlfn.CONCAT($K$20,": ",K23)</f>
         <v>Owner's Confirmation of Commitment: Health Authority</v>
       </c>
-      <c r="B22" t="s">
-        <v>78</v>
-      </c>
-      <c r="F22" t="str" cm="1">
-        <f t="array" aca="1" ref="F22" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J22),"$"))</f>
-        <v>J22</v>
-      </c>
-      <c r="G22">
+      <c r="B23" t="s">
+        <v>78</v>
+      </c>
+      <c r="D23">
+        <v>36</v>
+      </c>
+      <c r="E23">
+        <v>590</v>
+      </c>
+      <c r="F23" t="str" cm="1">
+        <f t="array" aca="1" ref="F23" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L23),"$"))</f>
+        <v>L23</v>
+      </c>
+      <c r="G23">
         <v>2</v>
       </c>
-      <c r="H22" t="s">
-        <v>123</v>
-      </c>
-      <c r="I22" s="5" t="s">
+      <c r="H23" t="s">
+        <v>123</v>
+      </c>
+      <c r="I23" t="s">
+        <v>126</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="J22" s="11" t="str">
-        <f>J2</f>
+      <c r="L23" s="11" t="str">
+        <f>L2</f>
         <v>Fraser</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" t="str">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I24" t="s">
+        <v>127</v>
+      </c>
+      <c r="J24">
+        <v>2</v>
+      </c>
+      <c r="K24" s="5"/>
+      <c r="L24" s="11"/>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A25" t="str">
         <f t="shared" si="3"/>
         <v>Owner's Confirmation of Commitment: Date</v>
       </c>
-      <c r="B23" t="s">
-        <v>78</v>
-      </c>
-      <c r="F23" t="str" cm="1">
-        <f t="array" aca="1" ref="F23" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J23),"$"))</f>
-        <v>J23</v>
-      </c>
-      <c r="G23">
+      <c r="B25" t="s">
+        <v>78</v>
+      </c>
+      <c r="D25">
+        <v>376</v>
+      </c>
+      <c r="E25">
+        <v>733</v>
+      </c>
+      <c r="F25" t="str" cm="1">
+        <f t="array" aca="1" ref="F25" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L25),"$"))</f>
+        <v>L25</v>
+      </c>
+      <c r="G25">
         <v>2</v>
       </c>
-      <c r="H23" t="s">
-        <v>123</v>
-      </c>
-      <c r="I23" s="6" t="s">
+      <c r="H25" t="s">
+        <v>123</v>
+      </c>
+      <c r="K25" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J23" s="12">
-        <f ca="1">J9</f>
-        <v>45949</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I24" s="20" t="s">
+      <c r="L25" s="12">
+        <f ca="1">L9</f>
+        <v>45957</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="K26" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="J24" s="20"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" t="str">
-        <f>_xlfn.CONCAT($I$24,": ",I25)</f>
+      <c r="L26" s="18"/>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A27" t="str">
+        <f>_xlfn.CONCAT($K$26,": ",K27)</f>
         <v>General Information: Name of Pool:</v>
       </c>
-      <c r="B25" t="s">
-        <v>78</v>
-      </c>
-      <c r="F25" t="str" cm="1">
-        <f t="array" aca="1" ref="F25" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J25),"$"))</f>
-        <v>J25</v>
-      </c>
-      <c r="G25">
+      <c r="B27" t="s">
+        <v>78</v>
+      </c>
+      <c r="D27">
+        <v>97</v>
+      </c>
+      <c r="E27">
+        <v>152</v>
+      </c>
+      <c r="F27" t="str" cm="1">
+        <f t="array" aca="1" ref="F27" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L27),"$"))</f>
+        <v>L27</v>
+      </c>
+      <c r="G27">
         <v>3</v>
       </c>
-      <c r="H25" t="s">
-        <v>123</v>
-      </c>
-      <c r="I25" s="5" t="s">
+      <c r="H27" t="s">
+        <v>123</v>
+      </c>
+      <c r="I27" t="s">
+        <v>127</v>
+      </c>
+      <c r="J27">
+        <v>9</v>
+      </c>
+      <c r="K27" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J25" s="2" t="str">
-        <f>J7</f>
+      <c r="L27" s="2" t="str">
+        <f>L7</f>
         <v>AME test pool</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" t="str">
-        <f t="shared" ref="A26:A27" si="4">_xlfn.CONCAT($I$24,": ",I26)</f>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A28" t="str">
+        <f t="shared" ref="A28:A29" si="4">_xlfn.CONCAT($K$26,": ",K28)</f>
         <v>General Information: Civic Address:</v>
       </c>
-      <c r="B26" t="s">
-        <v>78</v>
-      </c>
-      <c r="F26" t="str" cm="1">
-        <f t="array" aca="1" ref="F26" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J26),"$"))</f>
-        <v>J26</v>
-      </c>
-      <c r="G26">
+      <c r="B28" t="s">
+        <v>78</v>
+      </c>
+      <c r="D28">
+        <v>97</v>
+      </c>
+      <c r="E28">
+        <v>178</v>
+      </c>
+      <c r="F28" t="str" cm="1">
+        <f t="array" aca="1" ref="F28" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L28),"$"))</f>
+        <v>L28</v>
+      </c>
+      <c r="G28">
         <v>3</v>
       </c>
-      <c r="H26" t="s">
-        <v>123</v>
-      </c>
-      <c r="I26" s="6" t="s">
+      <c r="H28" t="s">
+        <v>123</v>
+      </c>
+      <c r="I28" t="s">
+        <v>127</v>
+      </c>
+      <c r="J28">
+        <v>9</v>
+      </c>
+      <c r="K28" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="J26" s="4" t="str">
-        <f>J8</f>
+      <c r="L28" s="4" t="str">
+        <f>L8</f>
         <v>1175 Douglas St #912, Victoria, BC V8W 2E1</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" t="str">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A29" t="str">
         <f t="shared" si="4"/>
         <v>General Information: Pool Type:</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B29" t="s">
         <v>79</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C29" t="s">
         <v>24</v>
       </c>
-      <c r="F27" t="str" cm="1">
-        <f t="array" aca="1" ref="F27" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J27),"$"))</f>
-        <v>J27</v>
-      </c>
-      <c r="G27">
+      <c r="D29">
+        <v>180</v>
+      </c>
+      <c r="E29">
+        <v>193</v>
+      </c>
+      <c r="F29" t="str" cm="1">
+        <f t="array" aca="1" ref="F29" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L29),"$"))</f>
+        <v>L29</v>
+      </c>
+      <c r="G29">
         <v>3</v>
       </c>
-      <c r="H27" t="s">
-        <v>123</v>
-      </c>
-      <c r="I27" s="5" t="s">
+      <c r="H29" t="s">
+        <v>123</v>
+      </c>
+      <c r="K29" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="J27" s="3" t="s">
+      <c r="L29" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C28" t="s">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="C30" t="s">
         <v>25</v>
       </c>
-      <c r="I28" s="5"/>
-      <c r="J28" s="3"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C29" t="s">
+      <c r="D30">
+        <v>282</v>
+      </c>
+      <c r="E30">
+        <v>193</v>
+      </c>
+      <c r="K30" s="5"/>
+      <c r="L30" s="3"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="C31" t="s">
         <v>26</v>
       </c>
-      <c r="I29" s="5"/>
-      <c r="J29" s="3"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C30" t="s">
+      <c r="D31">
+        <v>343</v>
+      </c>
+      <c r="E31">
+        <v>193</v>
+      </c>
+      <c r="K31" s="5"/>
+      <c r="L31" s="3"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="C32" t="s">
         <v>27</v>
       </c>
-      <c r="I30" s="5"/>
-      <c r="J30" s="3"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C31" t="s">
+      <c r="D32">
+        <v>414</v>
+      </c>
+      <c r="E32">
+        <v>193</v>
+      </c>
+      <c r="K32" s="5"/>
+      <c r="L32" s="3"/>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="C33" t="s">
         <v>28</v>
       </c>
-      <c r="I31" s="5"/>
-      <c r="J31" s="3"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" t="str">
-        <f>_xlfn.CONCAT($I$24,": ",I32)</f>
+      <c r="D33">
+        <v>497</v>
+      </c>
+      <c r="E33">
+        <v>193</v>
+      </c>
+      <c r="K33" s="5"/>
+      <c r="L33" s="3"/>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A34" t="str">
+        <f>_xlfn.CONCAT($K$26,": ",K34)</f>
         <v>General Information: Indoor/Outdoor</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B34" t="s">
         <v>79</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C34" t="s">
         <v>29</v>
       </c>
-      <c r="F32" t="str" cm="1">
-        <f t="array" aca="1" ref="F32" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J32),"$"))</f>
-        <v>J32</v>
-      </c>
-      <c r="G32">
+      <c r="D34">
+        <v>561</v>
+      </c>
+      <c r="E34">
+        <v>193</v>
+      </c>
+      <c r="F34" t="str" cm="1">
+        <f t="array" aca="1" ref="F34" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L34),"$"))</f>
+        <v>L34</v>
+      </c>
+      <c r="G34">
         <v>3</v>
       </c>
-      <c r="H32" t="s">
-        <v>123</v>
-      </c>
-      <c r="I32" s="6" t="s">
+      <c r="H34" t="s">
+        <v>123</v>
+      </c>
+      <c r="K34" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="J32" s="7" t="s">
+      <c r="L34" s="7" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C33" t="s">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="C35" t="s">
         <v>30</v>
       </c>
-      <c r="I33" s="6"/>
-      <c r="J33" s="7"/>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I34" s="20" t="s">
+      <c r="D35">
+        <v>561</v>
+      </c>
+      <c r="E35">
+        <v>204</v>
+      </c>
+      <c r="K35" s="6"/>
+      <c r="L35" s="7"/>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="K36" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="J34" s="20"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" t="str">
-        <f>_xlfn.CONCAT($I$34,": ",I35)</f>
+      <c r="L36" s="18"/>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A37" t="str">
+        <f>_xlfn.CONCAT($K$36,": ",K37)</f>
         <v>Owner Information: Name</v>
       </c>
-      <c r="B35" t="s">
-        <v>78</v>
-      </c>
-      <c r="F35" t="str" cm="1">
-        <f t="array" aca="1" ref="F35" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J35),"$"))</f>
-        <v>J35</v>
-      </c>
-      <c r="G35">
+      <c r="B37" t="s">
+        <v>78</v>
+      </c>
+      <c r="D37">
+        <v>144</v>
+      </c>
+      <c r="E37">
+        <v>253</v>
+      </c>
+      <c r="F37" t="str" cm="1">
+        <f t="array" aca="1" ref="F37" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L37),"$"))</f>
+        <v>L37</v>
+      </c>
+      <c r="G37">
         <v>3</v>
       </c>
-      <c r="H35" t="s">
-        <v>123</v>
-      </c>
-      <c r="I35" s="5" t="s">
+      <c r="H37" t="s">
+        <v>123</v>
+      </c>
+      <c r="I37" t="s">
+        <v>127</v>
+      </c>
+      <c r="J37">
+        <v>9</v>
+      </c>
+      <c r="K37" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="J35" s="3" t="s">
+      <c r="L37" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="K35" s="10" t="s">
+      <c r="M37" s="10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" t="str">
-        <f t="shared" ref="A36:A38" si="5">_xlfn.CONCAT($I$34,": ",I36)</f>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A38" t="str">
+        <f t="shared" ref="A38:A40" si="5">_xlfn.CONCAT($K$36,": ",K38)</f>
         <v>Owner Information: Address</v>
       </c>
-      <c r="B36" t="s">
-        <v>78</v>
-      </c>
-      <c r="F36" t="str" cm="1">
-        <f t="array" aca="1" ref="F36" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J36),"$"))</f>
-        <v>J36</v>
-      </c>
-      <c r="G36">
+      <c r="B38" t="s">
+        <v>78</v>
+      </c>
+      <c r="D38">
+        <v>73</v>
+      </c>
+      <c r="E38">
+        <v>279</v>
+      </c>
+      <c r="F38" t="str" cm="1">
+        <f t="array" aca="1" ref="F38" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L38),"$"))</f>
+        <v>L38</v>
+      </c>
+      <c r="G38">
         <v>3</v>
       </c>
-      <c r="H36" t="s">
-        <v>123</v>
-      </c>
-      <c r="I36" s="6" t="s">
+      <c r="H38" t="s">
+        <v>123</v>
+      </c>
+      <c r="I38" t="s">
+        <v>127</v>
+      </c>
+      <c r="J38">
+        <v>9</v>
+      </c>
+      <c r="K38" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="J36" s="7" t="s">
+      <c r="L38" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="K36" s="10" t="s">
+      <c r="M38" s="10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A37" t="str">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A39" t="str">
         <f t="shared" si="5"/>
         <v>Owner Information: Phone Number</v>
       </c>
-      <c r="B37" t="s">
-        <v>78</v>
-      </c>
-      <c r="F37" t="str" cm="1">
-        <f t="array" aca="1" ref="F37" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J37),"$"))</f>
-        <v>J37</v>
-      </c>
-      <c r="G37">
+      <c r="B39" t="s">
+        <v>78</v>
+      </c>
+      <c r="D39">
+        <v>104</v>
+      </c>
+      <c r="E39">
+        <v>306</v>
+      </c>
+      <c r="F39" t="str" cm="1">
+        <f t="array" aca="1" ref="F39" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L39),"$"))</f>
+        <v>L39</v>
+      </c>
+      <c r="G39">
         <v>3</v>
       </c>
-      <c r="H37" t="s">
-        <v>123</v>
-      </c>
-      <c r="I37" s="5" t="s">
+      <c r="H39" t="s">
+        <v>123</v>
+      </c>
+      <c r="I39" t="s">
+        <v>127</v>
+      </c>
+      <c r="J39">
+        <v>9</v>
+      </c>
+      <c r="K39" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="J37" s="3" t="s">
+      <c r="L39" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="K37" s="10" t="s">
+      <c r="M39" s="10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A38" t="str">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A40" t="str">
         <f t="shared" si="5"/>
         <v>Owner Information: Email</v>
       </c>
-      <c r="B38" t="s">
-        <v>78</v>
-      </c>
-      <c r="F38" t="str" cm="1">
-        <f t="array" aca="1" ref="F38" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J38),"$"))</f>
-        <v>J38</v>
-      </c>
-      <c r="G38">
-        <v>3</v>
-      </c>
-      <c r="H38" t="s">
-        <v>123</v>
-      </c>
-      <c r="I38" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="J38" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="K38" s="10" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I39" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="J39" s="20"/>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A40" t="str">
-        <f>_xlfn.CONCAT($I$39,": ",I40)</f>
-        <v>Designer Information (Append additional information for multiple designers): Name</v>
-      </c>
       <c r="B40" t="s">
         <v>78</v>
       </c>
+      <c r="D40">
+        <v>321</v>
+      </c>
+      <c r="E40">
+        <v>306</v>
+      </c>
       <c r="F40" t="str" cm="1">
-        <f t="array" aca="1" ref="F40" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J40),"$"))</f>
-        <v>J40</v>
+        <f t="array" aca="1" ref="F40" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L40),"$"))</f>
+        <v>L40</v>
       </c>
       <c r="G40">
         <v>3</v>
@@ -1788,60 +1983,86 @@
       <c r="H40" t="s">
         <v>123</v>
       </c>
-      <c r="I40" s="6" t="s">
+      <c r="I40" t="s">
+        <v>127</v>
+      </c>
+      <c r="J40">
+        <v>9</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="L40" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="M40" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="K41" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="L41" s="18"/>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A42" t="str">
+        <f>_xlfn.CONCAT($K$41,": ",K42)</f>
+        <v>Designer Information (Append additional information for multiple designers): Name</v>
+      </c>
+      <c r="B42" t="s">
+        <v>78</v>
+      </c>
+      <c r="D42">
+        <v>64</v>
+      </c>
+      <c r="E42">
+        <v>357</v>
+      </c>
+      <c r="F42" t="str" cm="1">
+        <f t="array" aca="1" ref="F42" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L42),"$"))</f>
+        <v>L42</v>
+      </c>
+      <c r="G42">
+        <v>3</v>
+      </c>
+      <c r="H42" t="s">
+        <v>123</v>
+      </c>
+      <c r="I42" t="s">
+        <v>127</v>
+      </c>
+      <c r="J42">
+        <v>10</v>
+      </c>
+      <c r="K42" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="J40" s="4" t="str">
-        <f>J16</f>
+      <c r="L42" s="4" t="str">
+        <f>L16</f>
         <v>John Doe</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A41" t="str">
-        <f>_xlfn.CONCAT($I$39,": ",I41)</f>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A43" t="str">
+        <f>_xlfn.CONCAT($K$41,": ",K43)</f>
         <v>Designer Information (Append additional information for multiple designers): Professional Designation</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B43" t="s">
         <v>79</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C43" t="s">
         <v>43</v>
       </c>
-      <c r="F41" t="str" cm="1">
-        <f t="array" aca="1" ref="F41" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J41),"$"))</f>
-        <v>J41</v>
-      </c>
-      <c r="G41">
-        <v>3</v>
-      </c>
-      <c r="H41" t="s">
-        <v>123</v>
-      </c>
-      <c r="I41" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="J41" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C42" t="s">
-        <v>81</v>
-      </c>
-      <c r="I42" s="5"/>
-      <c r="J42" s="3"/>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A43" t="str">
-        <f t="shared" ref="A43:A46" si="6">_xlfn.CONCAT($I$39,": ",I43)</f>
-        <v>Designer Information (Append additional information for multiple designers): Company (Legal Corporate)</v>
-      </c>
-      <c r="B43" t="s">
-        <v>78</v>
+      <c r="D43">
+        <v>516</v>
+      </c>
+      <c r="E43">
+        <v>343</v>
       </c>
       <c r="F43" t="str" cm="1">
-        <f t="array" aca="1" ref="F43" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J43),"$"))</f>
-        <v>J43</v>
+        <f t="array" aca="1" ref="F43" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L43),"$"))</f>
+        <v>L43</v>
       </c>
       <c r="G43">
         <v>3</v>
@@ -1849,108 +2070,156 @@
       <c r="H43" t="s">
         <v>123</v>
       </c>
-      <c r="I43" s="6" t="s">
+      <c r="K43" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="L43" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="C44" t="s">
+        <v>81</v>
+      </c>
+      <c r="D44">
+        <v>516</v>
+      </c>
+      <c r="E44">
+        <v>354</v>
+      </c>
+      <c r="K44" s="5"/>
+      <c r="L44" s="3"/>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A45" t="str">
+        <f t="shared" ref="A45:A48" si="6">_xlfn.CONCAT($K$41,": ",K45)</f>
+        <v>Designer Information (Append additional information for multiple designers): Company (Legal Corporate)</v>
+      </c>
+      <c r="B45" t="s">
+        <v>78</v>
+      </c>
+      <c r="D45">
+        <v>161</v>
+      </c>
+      <c r="E45">
+        <v>383</v>
+      </c>
+      <c r="F45" t="str" cm="1">
+        <f t="array" aca="1" ref="F45" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L45),"$"))</f>
+        <v>L45</v>
+      </c>
+      <c r="G45">
+        <v>3</v>
+      </c>
+      <c r="H45" t="s">
+        <v>123</v>
+      </c>
+      <c r="I45" t="s">
+        <v>127</v>
+      </c>
+      <c r="J45">
+        <v>10</v>
+      </c>
+      <c r="K45" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="J43" s="7" t="s">
+      <c r="L45" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A44" t="str">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A46" t="str">
         <f t="shared" si="6"/>
         <v>Designer Information (Append additional information for multiple designers): Address</v>
       </c>
-      <c r="B44" t="s">
-        <v>78</v>
-      </c>
-      <c r="F44" t="str" cm="1">
-        <f t="array" aca="1" ref="F44" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J44),"$"))</f>
-        <v>J44</v>
-      </c>
-      <c r="G44">
+      <c r="B46" t="s">
+        <v>78</v>
+      </c>
+      <c r="D46">
+        <v>73</v>
+      </c>
+      <c r="E46">
+        <v>409</v>
+      </c>
+      <c r="F46" t="str" cm="1">
+        <f t="array" aca="1" ref="F46" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L46),"$"))</f>
+        <v>L46</v>
+      </c>
+      <c r="G46">
         <v>3</v>
       </c>
-      <c r="H44" t="s">
-        <v>123</v>
-      </c>
-      <c r="I44" s="5" t="s">
+      <c r="H46" t="s">
+        <v>123</v>
+      </c>
+      <c r="I46" t="s">
+        <v>127</v>
+      </c>
+      <c r="J46">
+        <v>10</v>
+      </c>
+      <c r="K46" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="J44" s="2" t="str">
-        <f>J17</f>
+      <c r="L46" s="2" t="str">
+        <f>L17</f>
         <v>638 Smithe St Suite 200, Vancouver, BC V6B 1E3</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A45" t="str">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A47" t="str">
         <f t="shared" si="6"/>
         <v>Designer Information (Append additional information for multiple designers): Phone Number</v>
       </c>
-      <c r="B45" t="s">
-        <v>78</v>
-      </c>
-      <c r="F45" t="str" cm="1">
-        <f t="array" aca="1" ref="F45" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J45),"$"))</f>
-        <v>J45</v>
-      </c>
-      <c r="G45">
+      <c r="B47" t="s">
+        <v>78</v>
+      </c>
+      <c r="D47">
+        <v>104</v>
+      </c>
+      <c r="E47">
+        <v>435</v>
+      </c>
+      <c r="F47" t="str" cm="1">
+        <f t="array" aca="1" ref="F47" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L47),"$"))</f>
+        <v>L47</v>
+      </c>
+      <c r="G47">
         <v>3</v>
       </c>
-      <c r="H45" t="s">
-        <v>123</v>
-      </c>
-      <c r="I45" s="6" t="s">
+      <c r="H47" t="s">
+        <v>123</v>
+      </c>
+      <c r="I47" t="s">
+        <v>127</v>
+      </c>
+      <c r="J47">
+        <v>10</v>
+      </c>
+      <c r="K47" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="J45" s="4" t="str">
-        <f>J18</f>
+      <c r="L47" s="4" t="str">
+        <f>L18</f>
         <v>098-765-4321</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A46" t="str">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A48" t="str">
         <f t="shared" si="6"/>
         <v>Designer Information (Append additional information for multiple designers): Email</v>
       </c>
-      <c r="B46" t="s">
-        <v>78</v>
-      </c>
-      <c r="F46" t="str" cm="1">
-        <f t="array" aca="1" ref="F46" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J46),"$"))</f>
-        <v>J46</v>
-      </c>
-      <c r="G46">
-        <v>3</v>
-      </c>
-      <c r="H46" t="s">
-        <v>123</v>
-      </c>
-      <c r="I46" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="J46" s="2" t="str">
-        <f>J19</f>
-        <v>random@icould.com</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I47" s="20" t="s">
-        <v>44</v>
-      </c>
-      <c r="J47" s="20"/>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A48" t="str">
-        <f>_xlfn.CONCAT($I$47,": ",I48)</f>
-        <v>General Pool Parameters: Pool Volume: (m^3)</v>
-      </c>
       <c r="B48" t="s">
         <v>78</v>
       </c>
+      <c r="D48">
+        <v>321</v>
+      </c>
+      <c r="E48">
+        <v>435</v>
+      </c>
       <c r="F48" t="str" cm="1">
-        <f t="array" aca="1" ref="F48" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J48),"$"))</f>
-        <v>J48</v>
+        <f t="array" aca="1" ref="F48" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L48),"$"))</f>
+        <v>L48</v>
       </c>
       <c r="G48">
         <v>3</v>
@@ -1958,316 +2227,457 @@
       <c r="H48" t="s">
         <v>123</v>
       </c>
-      <c r="I48" s="5" t="s">
+      <c r="I48" t="s">
+        <v>127</v>
+      </c>
+      <c r="J48">
+        <v>10</v>
+      </c>
+      <c r="K48" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L48" s="2" t="str">
+        <f>L19</f>
+        <v>random@icould.com</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="K49" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="L49" s="18"/>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A50" t="str">
+        <f>_xlfn.CONCAT($K$49,": ",K50)</f>
+        <v>General Pool Parameters: Pool Volume: (m^3)</v>
+      </c>
+      <c r="B50" t="s">
+        <v>78</v>
+      </c>
+      <c r="D50">
+        <v>115</v>
+      </c>
+      <c r="E50">
+        <v>491</v>
+      </c>
+      <c r="F50" t="str" cm="1">
+        <f t="array" aca="1" ref="F50" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L50),"$"))</f>
+        <v>L50</v>
+      </c>
+      <c r="G50">
+        <v>3</v>
+      </c>
+      <c r="H50" t="s">
+        <v>123</v>
+      </c>
+      <c r="I50" t="s">
+        <v>127</v>
+      </c>
+      <c r="J50">
+        <v>11</v>
+      </c>
+      <c r="K50" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="J48" s="13">
+      <c r="L50" s="13">
         <v>300</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A49" t="str">
-        <f t="shared" ref="A49:A59" si="7">_xlfn.CONCAT($I$47,": ",I49)</f>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A51" t="str">
+        <f t="shared" ref="A51:A61" si="7">_xlfn.CONCAT($K$49,": ",K51)</f>
         <v>General Pool Parameters: Turnover: (hours)</v>
       </c>
-      <c r="B49" t="s">
-        <v>78</v>
-      </c>
-      <c r="F49" t="str" cm="1">
-        <f t="array" aca="1" ref="F49" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J49),"$"))</f>
-        <v>J49</v>
-      </c>
-      <c r="G49">
+      <c r="B51" t="s">
+        <v>78</v>
+      </c>
+      <c r="D51">
+        <v>232</v>
+      </c>
+      <c r="E51">
+        <v>491</v>
+      </c>
+      <c r="F51" t="str" cm="1">
+        <f t="array" aca="1" ref="F51" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L51),"$"))</f>
+        <v>L51</v>
+      </c>
+      <c r="G51">
         <v>3</v>
       </c>
-      <c r="H49" t="s">
-        <v>123</v>
-      </c>
-      <c r="I49" s="6" t="s">
+      <c r="H51" t="s">
+        <v>123</v>
+      </c>
+      <c r="I51" t="s">
+        <v>127</v>
+      </c>
+      <c r="J51">
+        <v>11</v>
+      </c>
+      <c r="K51" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="J49" s="14">
+      <c r="L51" s="14">
         <v>2.33</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A50" t="str">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A52" t="str">
         <f t="shared" si="7"/>
         <v>General Pool Parameters: Design Re-circulation Flow Rate: (L/sec)</v>
       </c>
-      <c r="B50" t="s">
-        <v>78</v>
-      </c>
-      <c r="F50" t="str" cm="1">
-        <f t="array" aca="1" ref="F50" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J50),"$"))</f>
-        <v>J50</v>
-      </c>
-      <c r="G50">
+      <c r="B52" t="s">
+        <v>78</v>
+      </c>
+      <c r="D52">
+        <v>468</v>
+      </c>
+      <c r="E52">
+        <v>491</v>
+      </c>
+      <c r="F52" t="str" cm="1">
+        <f t="array" aca="1" ref="F52" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L52),"$"))</f>
+        <v>L52</v>
+      </c>
+      <c r="G52">
         <v>3</v>
       </c>
-      <c r="H50" t="s">
-        <v>123</v>
-      </c>
-      <c r="I50" s="5" t="s">
+      <c r="H52" t="s">
+        <v>123</v>
+      </c>
+      <c r="I52" t="s">
+        <v>127</v>
+      </c>
+      <c r="J52">
+        <v>11</v>
+      </c>
+      <c r="K52" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="J50" s="13">
+      <c r="L52" s="13">
         <v>1200</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A51" t="str">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A53" t="str">
         <f t="shared" si="7"/>
         <v>General Pool Parameters: Pool Area (m^2)</v>
       </c>
-      <c r="B51" t="s">
-        <v>78</v>
-      </c>
-      <c r="F51" t="str" cm="1">
-        <f t="array" aca="1" ref="F51" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J51),"$"))</f>
-        <v>J51</v>
-      </c>
-      <c r="G51">
+      <c r="B53" t="s">
+        <v>78</v>
+      </c>
+      <c r="D53">
+        <v>148</v>
+      </c>
+      <c r="E53">
+        <v>522</v>
+      </c>
+      <c r="F53" t="str" cm="1">
+        <f t="array" aca="1" ref="F53" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L53),"$"))</f>
+        <v>L53</v>
+      </c>
+      <c r="G53">
         <v>3</v>
       </c>
-      <c r="H51" t="s">
-        <v>123</v>
-      </c>
-      <c r="I51" s="6" t="s">
+      <c r="H53" t="s">
+        <v>123</v>
+      </c>
+      <c r="I53" t="s">
+        <v>127</v>
+      </c>
+      <c r="J53">
+        <v>11</v>
+      </c>
+      <c r="K53" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J51" s="14">
+      <c r="L53" s="14">
         <v>30</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A52" t="str">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A54" t="str">
         <f t="shared" si="7"/>
         <v>General Pool Parameters: Deck Area (m^2)</v>
       </c>
-      <c r="B52" t="s">
-        <v>78</v>
-      </c>
-      <c r="F52" t="str" cm="1">
-        <f t="array" aca="1" ref="F52" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J52),"$"))</f>
-        <v>J52</v>
-      </c>
-      <c r="G52">
+      <c r="B54" t="s">
+        <v>78</v>
+      </c>
+      <c r="D54">
+        <v>243</v>
+      </c>
+      <c r="E54">
+        <v>522</v>
+      </c>
+      <c r="F54" t="str" cm="1">
+        <f t="array" aca="1" ref="F54" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L54),"$"))</f>
+        <v>L54</v>
+      </c>
+      <c r="G54">
         <v>3</v>
       </c>
-      <c r="H52" t="s">
-        <v>123</v>
-      </c>
-      <c r="I52" s="5" t="s">
+      <c r="H54" t="s">
+        <v>123</v>
+      </c>
+      <c r="I54" t="s">
+        <v>127</v>
+      </c>
+      <c r="J54">
+        <v>11</v>
+      </c>
+      <c r="K54" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="J52" s="13">
+      <c r="L54" s="13">
         <v>20</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A53" t="str">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A55" t="str">
         <f t="shared" si="7"/>
         <v>General Pool Parameters: Minimum Water Depth</v>
       </c>
-      <c r="B53" t="s">
-        <v>78</v>
-      </c>
-      <c r="F53" t="str" cm="1">
-        <f t="array" aca="1" ref="F53" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J53),"$"))</f>
-        <v>J53</v>
-      </c>
-      <c r="G53">
+      <c r="B55" t="s">
+        <v>78</v>
+      </c>
+      <c r="D55">
+        <v>420</v>
+      </c>
+      <c r="E55">
+        <v>522</v>
+      </c>
+      <c r="F55" t="str" cm="1">
+        <f t="array" aca="1" ref="F55" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L55),"$"))</f>
+        <v>L55</v>
+      </c>
+      <c r="G55">
         <v>3</v>
       </c>
-      <c r="H53" t="s">
-        <v>123</v>
-      </c>
-      <c r="I53" s="6" t="s">
+      <c r="H55" t="s">
+        <v>123</v>
+      </c>
+      <c r="I55" t="s">
+        <v>127</v>
+      </c>
+      <c r="J55">
+        <v>11</v>
+      </c>
+      <c r="K55" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="J53" s="14">
+      <c r="L55" s="14">
         <v>1</v>
       </c>
-      <c r="K53" s="10" t="s">
+      <c r="M55" s="10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A54" t="str">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A56" t="str">
         <f t="shared" si="7"/>
         <v>General Pool Parameters: Maximum Water Depth</v>
       </c>
-      <c r="B54" t="s">
-        <v>78</v>
-      </c>
-      <c r="F54" t="str" cm="1">
-        <f t="array" aca="1" ref="F54" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J54),"$"))</f>
-        <v>J54</v>
-      </c>
-      <c r="G54">
+      <c r="B56" t="s">
+        <v>78</v>
+      </c>
+      <c r="D56">
+        <v>515</v>
+      </c>
+      <c r="E56">
+        <v>522</v>
+      </c>
+      <c r="F56" t="str" cm="1">
+        <f t="array" aca="1" ref="F56" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L56),"$"))</f>
+        <v>L56</v>
+      </c>
+      <c r="G56">
         <v>3</v>
       </c>
-      <c r="H54" t="s">
-        <v>123</v>
-      </c>
-      <c r="I54" s="5" t="s">
+      <c r="H56" t="s">
+        <v>123</v>
+      </c>
+      <c r="I56" t="s">
+        <v>127</v>
+      </c>
+      <c r="J56">
+        <v>11</v>
+      </c>
+      <c r="K56" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="J54" s="13">
+      <c r="L56" s="13">
         <v>3</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A55" t="str">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A57" t="str">
         <f t="shared" si="7"/>
         <v>General Pool Parameters: Shallow Bathing Load</v>
       </c>
-      <c r="B55" t="s">
-        <v>78</v>
-      </c>
-      <c r="F55" t="str" cm="1">
-        <f t="array" aca="1" ref="F55" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J55),"$"))</f>
-        <v>J55</v>
-      </c>
-      <c r="G55">
+      <c r="B57" t="s">
+        <v>78</v>
+      </c>
+      <c r="D57">
+        <v>163</v>
+      </c>
+      <c r="E57">
+        <v>552</v>
+      </c>
+      <c r="F57" t="str" cm="1">
+        <f t="array" aca="1" ref="F57" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L57),"$"))</f>
+        <v>L57</v>
+      </c>
+      <c r="G57">
         <v>3</v>
       </c>
-      <c r="H55" t="s">
-        <v>123</v>
-      </c>
-      <c r="I55" s="6" t="s">
+      <c r="H57" t="s">
+        <v>123</v>
+      </c>
+      <c r="I57" t="s">
+        <v>127</v>
+      </c>
+      <c r="J57">
+        <v>11</v>
+      </c>
+      <c r="K57" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="J55" s="14">
+      <c r="L57" s="14">
         <v>100</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A56" t="str">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A58" t="str">
         <f t="shared" si="7"/>
         <v>General Pool Parameters: Deep Bathing Load</v>
       </c>
-      <c r="B56" t="s">
-        <v>78</v>
-      </c>
-      <c r="F56" t="str" cm="1">
-        <f t="array" aca="1" ref="F56" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J56),"$"))</f>
-        <v>J56</v>
-      </c>
-      <c r="G56">
+      <c r="B58" t="s">
+        <v>78</v>
+      </c>
+      <c r="D58">
+        <v>315</v>
+      </c>
+      <c r="E58">
+        <v>552</v>
+      </c>
+      <c r="F58" t="str" cm="1">
+        <f t="array" aca="1" ref="F58" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L58),"$"))</f>
+        <v>L58</v>
+      </c>
+      <c r="G58">
         <v>3</v>
       </c>
-      <c r="H56" t="s">
-        <v>123</v>
-      </c>
-      <c r="I56" s="5" t="s">
+      <c r="H58" t="s">
+        <v>123</v>
+      </c>
+      <c r="I58" t="s">
+        <v>127</v>
+      </c>
+      <c r="J58">
+        <v>11</v>
+      </c>
+      <c r="K58" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="J56" s="13">
+      <c r="L58" s="13">
         <v>100</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A57" t="str">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A59" t="str">
         <f t="shared" si="7"/>
         <v>General Pool Parameters: Total Bathing Load</v>
       </c>
-      <c r="B57" t="s">
-        <v>78</v>
-      </c>
-      <c r="F57" t="str" cm="1">
-        <f t="array" aca="1" ref="F57" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J57),"$"))</f>
-        <v>J57</v>
-      </c>
-      <c r="G57">
+      <c r="B59" t="s">
+        <v>78</v>
+      </c>
+      <c r="D59">
+        <v>469</v>
+      </c>
+      <c r="E59">
+        <v>552</v>
+      </c>
+      <c r="F59" t="str" cm="1">
+        <f t="array" aca="1" ref="F59" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L59),"$"))</f>
+        <v>L59</v>
+      </c>
+      <c r="G59">
         <v>3</v>
       </c>
-      <c r="H57" t="s">
-        <v>123</v>
-      </c>
-      <c r="I57" s="6" t="s">
+      <c r="H59" t="s">
+        <v>123</v>
+      </c>
+      <c r="I59" t="s">
+        <v>127</v>
+      </c>
+      <c r="J59">
+        <v>11</v>
+      </c>
+      <c r="K59" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="J57" s="15">
-        <f>SUM(J55:J56)</f>
+      <c r="L59" s="15">
+        <f>SUM(L57:L58)</f>
         <v>200</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A58" t="str">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A60" t="str">
         <f t="shared" si="7"/>
         <v>General Pool Parameters: Pool Basin Color</v>
       </c>
-      <c r="B58" t="s">
-        <v>78</v>
-      </c>
-      <c r="F58" t="str" cm="1">
-        <f t="array" aca="1" ref="F58" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J58),"$"))</f>
-        <v>J58</v>
-      </c>
-      <c r="G58">
+      <c r="B60" t="s">
+        <v>78</v>
+      </c>
+      <c r="D60">
+        <v>157</v>
+      </c>
+      <c r="E60">
+        <v>582</v>
+      </c>
+      <c r="F60" t="str" cm="1">
+        <f t="array" aca="1" ref="F60" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L60),"$"))</f>
+        <v>L60</v>
+      </c>
+      <c r="G60">
         <v>3</v>
       </c>
-      <c r="H58" t="s">
-        <v>123</v>
-      </c>
-      <c r="I58" s="5" t="s">
+      <c r="H60" t="s">
+        <v>123</v>
+      </c>
+      <c r="I60" t="s">
+        <v>127</v>
+      </c>
+      <c r="J60">
+        <v>11</v>
+      </c>
+      <c r="K60" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="J58" s="13" t="s">
+      <c r="L60" s="13" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A59" t="str">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A61" t="str">
         <f t="shared" si="7"/>
         <v>General Pool Parameters: Complies with Pool Regulations</v>
       </c>
-      <c r="B59" t="s">
-        <v>79</v>
-      </c>
-      <c r="C59" t="s">
-        <v>57</v>
-      </c>
-      <c r="F59" t="str" cm="1">
-        <f t="array" aca="1" ref="F59" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J59),"$"))</f>
-        <v>J59</v>
-      </c>
-      <c r="G59">
-        <v>3</v>
-      </c>
-      <c r="H59" t="s">
-        <v>123</v>
-      </c>
-      <c r="I59" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="J59" s="14" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C60" t="s">
-        <v>58</v>
-      </c>
-      <c r="I60" s="6"/>
-      <c r="J60" s="14"/>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A61" t="str">
-        <f t="shared" ref="A61:A68" si="8">_xlfn.CONCAT($I$47,": ",I61)</f>
-        <v>General Pool Parameters: Filters</v>
-      </c>
       <c r="B61" t="s">
         <v>79</v>
       </c>
       <c r="C61" t="s">
-        <v>61</v>
+        <v>57</v>
+      </c>
+      <c r="D61">
+        <v>444</v>
+      </c>
+      <c r="E61">
+        <v>568</v>
       </c>
       <c r="F61" t="str" cm="1">
-        <f t="array" aca="1" ref="F61" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J61),"$"))</f>
-        <v>J61</v>
+        <f t="array" aca="1" ref="F61" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L61),"$"))</f>
+        <v>L61</v>
       </c>
       <c r="G61">
         <v>3</v>
@@ -2275,137 +2685,170 @@
       <c r="H61" t="s">
         <v>123</v>
       </c>
-      <c r="I61" s="5" t="s">
+      <c r="K61" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="L61" s="14" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="C62" t="s">
+        <v>58</v>
+      </c>
+      <c r="D62">
+        <v>481</v>
+      </c>
+      <c r="E62">
+        <v>568</v>
+      </c>
+      <c r="K62" s="6"/>
+      <c r="L62" s="14"/>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A63" t="str">
+        <f t="shared" ref="A63:A70" si="8">_xlfn.CONCAT($K$49,": ",K63)</f>
+        <v>General Pool Parameters: Filters</v>
+      </c>
+      <c r="B63" t="s">
+        <v>79</v>
+      </c>
+      <c r="C63" t="s">
+        <v>61</v>
+      </c>
+      <c r="D63">
+        <v>154</v>
+      </c>
+      <c r="E63">
+        <v>597</v>
+      </c>
+      <c r="F63" t="str" cm="1">
+        <f t="array" aca="1" ref="F63" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L63),"$"))</f>
+        <v>L63</v>
+      </c>
+      <c r="G63">
+        <v>3</v>
+      </c>
+      <c r="H63" t="s">
+        <v>123</v>
+      </c>
+      <c r="K63" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="J61" s="13" t="s">
+      <c r="L63" s="13" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C62" t="s">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="C64" t="s">
         <v>76</v>
       </c>
-      <c r="I62" s="5"/>
-      <c r="J62" s="13"/>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C63" t="s">
+      <c r="D64">
+        <v>201</v>
+      </c>
+      <c r="E64">
+        <v>597</v>
+      </c>
+      <c r="K64" s="5"/>
+      <c r="L64" s="13"/>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C65" t="s">
         <v>62</v>
       </c>
-      <c r="I63" s="5"/>
-      <c r="J63" s="13"/>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C64" t="s">
+      <c r="D65">
+        <v>270</v>
+      </c>
+      <c r="E65">
+        <v>597</v>
+      </c>
+      <c r="K65" s="5"/>
+      <c r="L65" s="13"/>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C66" t="s">
         <v>63</v>
       </c>
-      <c r="I64" s="5"/>
-      <c r="J64" s="13"/>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C65" t="s">
+      <c r="D66">
+        <v>338</v>
+      </c>
+      <c r="E66">
+        <v>597</v>
+      </c>
+      <c r="K66" s="5"/>
+      <c r="L66" s="13"/>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C67" t="s">
         <v>64</v>
       </c>
-      <c r="I65" s="5"/>
-      <c r="J65" s="13"/>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A66" t="str">
+      <c r="D67">
+        <v>398</v>
+      </c>
+      <c r="E67">
+        <v>597</v>
+      </c>
+      <c r="K67" s="5"/>
+      <c r="L67" s="13"/>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A68" t="str">
         <f t="shared" si="8"/>
         <v>General Pool Parameters: NSF Approved</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B68" t="s">
         <v>79</v>
       </c>
-      <c r="C66" t="s">
+      <c r="C68" t="s">
         <v>57</v>
       </c>
-      <c r="F66" t="str" cm="1">
-        <f t="array" aca="1" ref="F66" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J66),"$"))</f>
-        <v>J66</v>
-      </c>
-      <c r="G66">
+      <c r="D68">
+        <v>537</v>
+      </c>
+      <c r="E68">
+        <v>597</v>
+      </c>
+      <c r="F68" t="str" cm="1">
+        <f t="array" aca="1" ref="F68" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L68),"$"))</f>
+        <v>L68</v>
+      </c>
+      <c r="G68">
         <v>3</v>
       </c>
-      <c r="H66" t="s">
-        <v>123</v>
-      </c>
-      <c r="I66" s="6" t="s">
+      <c r="H68" t="s">
+        <v>123</v>
+      </c>
+      <c r="K68" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="J66" s="14" t="s">
+      <c r="L68" s="14" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C67" t="s">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C69" t="s">
         <v>58</v>
       </c>
-      <c r="I67" s="6"/>
-      <c r="J67" s="14"/>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A68" t="str">
+      <c r="D69">
+        <v>567</v>
+      </c>
+      <c r="E69">
+        <v>597</v>
+      </c>
+      <c r="K69" s="6"/>
+      <c r="L69" s="14"/>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A70" t="str">
         <f t="shared" si="8"/>
         <v>General Pool Parameters: Pressure Gauge Quantity</v>
       </c>
-      <c r="B68" t="s">
-        <v>78</v>
-      </c>
-      <c r="F68" t="str" cm="1">
-        <f t="array" aca="1" ref="F68" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J68),"$"))</f>
-        <v>J68</v>
-      </c>
-      <c r="G68">
-        <v>3</v>
-      </c>
-      <c r="H68" t="s">
-        <v>123</v>
-      </c>
-      <c r="I68" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="J68" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A69" t="str">
-        <f>_xlfn.CONCAT($I$47,": ",I69)</f>
-        <v>General Pool Parameters: Vacuum Gauge Quantity</v>
-      </c>
-      <c r="B69" t="s">
-        <v>78</v>
-      </c>
-      <c r="F69" t="str" cm="1">
-        <f t="array" aca="1" ref="F69" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J69),"$"))</f>
-        <v>J69</v>
-      </c>
-      <c r="G69">
-        <v>3</v>
-      </c>
-      <c r="H69" t="s">
-        <v>123</v>
-      </c>
-      <c r="I69" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="J69" s="14">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A70" t="str">
-        <f>_xlfn.CONCAT($I$47,": ",I70)</f>
-        <v>General Pool Parameters: Temperature Gauge Quantity</v>
-      </c>
       <c r="B70" t="s">
         <v>78</v>
       </c>
       <c r="F70" t="str" cm="1">
-        <f t="array" aca="1" ref="F70" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J70),"$"))</f>
-        <v>J70</v>
+        <f t="array" aca="1" ref="F70" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L70),"$"))</f>
+        <v>L70</v>
       </c>
       <c r="G70">
         <v>3</v>
@@ -2413,27 +2856,24 @@
       <c r="H70" t="s">
         <v>123</v>
       </c>
-      <c r="I70" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="J70" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K70" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="L70" s="13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A71" t="str">
-        <f>_xlfn.CONCAT($I$47,": ",I71)</f>
-        <v>General Pool Parameters: Disinfection</v>
+        <f>_xlfn.CONCAT($K$49,": ",K71)</f>
+        <v>General Pool Parameters: Vacuum Gauge Quantity</v>
       </c>
       <c r="B71" t="s">
-        <v>79</v>
-      </c>
-      <c r="C71" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="F71" t="str" cm="1">
-        <f t="array" aca="1" ref="F71" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J71),"$"))</f>
-        <v>J71</v>
+        <f t="array" aca="1" ref="F71" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L71),"$"))</f>
+        <v>L71</v>
       </c>
       <c r="G71">
         <v>3</v>
@@ -2441,119 +2881,141 @@
       <c r="H71" t="s">
         <v>123</v>
       </c>
-      <c r="I71" s="6" t="s">
+      <c r="K71" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="L71" s="14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A72" t="str">
+        <f>_xlfn.CONCAT($K$49,": ",K72)</f>
+        <v>General Pool Parameters: Temperature Gauge Quantity</v>
+      </c>
+      <c r="B72" t="s">
+        <v>78</v>
+      </c>
+      <c r="F72" t="str" cm="1">
+        <f t="array" aca="1" ref="F72" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L72),"$"))</f>
+        <v>L72</v>
+      </c>
+      <c r="G72">
+        <v>3</v>
+      </c>
+      <c r="H72" t="s">
+        <v>123</v>
+      </c>
+      <c r="K72" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="L72" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A73" t="str">
+        <f>_xlfn.CONCAT($K$49,": ",K73)</f>
+        <v>General Pool Parameters: Disinfection</v>
+      </c>
+      <c r="B73" t="s">
+        <v>79</v>
+      </c>
+      <c r="C73" t="s">
+        <v>70</v>
+      </c>
+      <c r="F73" t="str" cm="1">
+        <f t="array" aca="1" ref="F73" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L73),"$"))</f>
+        <v>L73</v>
+      </c>
+      <c r="G73">
+        <v>3</v>
+      </c>
+      <c r="H73" t="s">
+        <v>123</v>
+      </c>
+      <c r="K73" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="J71" s="14" t="s">
+      <c r="L73" s="14" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C72" t="s">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C74" t="s">
         <v>71</v>
       </c>
-      <c r="I72" s="6"/>
-      <c r="J72" s="14"/>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C73" t="s">
+      <c r="K74" s="6"/>
+      <c r="L74" s="14"/>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C75" t="s">
         <v>72</v>
       </c>
-      <c r="I73" s="6"/>
-      <c r="J73" s="14"/>
-    </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C74" t="s">
+      <c r="K75" s="6"/>
+      <c r="L75" s="14"/>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C76" t="s">
         <v>73</v>
       </c>
-      <c r="I74" s="6"/>
-      <c r="J74" s="14"/>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C75" t="s">
+      <c r="K76" s="6"/>
+      <c r="L76" s="14"/>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C77" t="s">
         <v>74</v>
       </c>
-      <c r="I75" s="6"/>
-      <c r="J75" s="14"/>
-    </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I76" s="20" t="s">
+      <c r="K77" s="6"/>
+      <c r="L77" s="14"/>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K78" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="J76" s="20"/>
-    </row>
-    <row r="77" spans="1:10" ht="90" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+      <c r="L78" s="18"/>
+    </row>
+    <row r="79" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
         <v>84</v>
       </c>
-      <c r="B77" t="s">
+      <c r="B79" t="s">
         <v>79</v>
       </c>
-      <c r="C77" t="s">
+      <c r="C79" t="s">
         <v>57</v>
       </c>
-      <c r="F77" t="str" cm="1">
-        <f t="array" aca="1" ref="F77" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J77),"$"))</f>
-        <v>J77</v>
-      </c>
-      <c r="G77">
+      <c r="F79" t="str" cm="1">
+        <f t="array" aca="1" ref="F79" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L79),"$"))</f>
+        <v>L79</v>
+      </c>
+      <c r="G79">
         <v>4</v>
       </c>
-      <c r="I77" s="17" t="s">
+      <c r="K79" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="J77" s="13" t="s">
+      <c r="L79" s="13" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C78" t="s">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C80" t="s">
         <v>58</v>
       </c>
-      <c r="I78" s="5"/>
-      <c r="J78" s="13"/>
-    </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C79" t="s">
+      <c r="K80" s="5"/>
+      <c r="L80" s="13"/>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C81" t="s">
         <v>85</v>
       </c>
-      <c r="I79" s="5"/>
-      <c r="J79" s="13"/>
-    </row>
-    <row r="80" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
+      <c r="K81" s="5"/>
+      <c r="L81" s="13"/>
+    </row>
+    <row r="82" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
         <v>86</v>
-      </c>
-      <c r="B80" t="s">
-        <v>79</v>
-      </c>
-      <c r="C80" t="s">
-        <v>57</v>
-      </c>
-      <c r="F80" t="str" cm="1">
-        <f t="array" aca="1" ref="F80" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J80),"$"))</f>
-        <v>J80</v>
-      </c>
-      <c r="G80">
-        <v>4</v>
-      </c>
-      <c r="I80" s="18" t="s">
-        <v>87</v>
-      </c>
-      <c r="J80" s="14" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C81" t="s">
-        <v>58</v>
-      </c>
-      <c r="I81" s="6"/>
-      <c r="J81" s="14"/>
-    </row>
-    <row r="82" spans="1:10" ht="60" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>88</v>
       </c>
       <c r="B82" t="s">
         <v>79</v>
@@ -2562,29 +3024,29 @@
         <v>57</v>
       </c>
       <c r="F82" t="str" cm="1">
-        <f t="array" aca="1" ref="F82" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J82),"$"))</f>
-        <v>J82</v>
+        <f t="array" aca="1" ref="F82" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L82),"$"))</f>
+        <v>L82</v>
       </c>
       <c r="G82">
         <v>4</v>
       </c>
-      <c r="I82" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="J82" s="13" t="s">
+      <c r="K82" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="L82" s="14" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C83" t="s">
         <v>58</v>
       </c>
-      <c r="I83" s="5"/>
-      <c r="J83" s="13"/>
-    </row>
-    <row r="84" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="K83" s="6"/>
+      <c r="L83" s="14"/>
+    </row>
+    <row r="84" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B84" t="s">
         <v>79</v>
@@ -2593,29 +3055,29 @@
         <v>57</v>
       </c>
       <c r="F84" t="str" cm="1">
-        <f t="array" aca="1" ref="F84" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J84),"$"))</f>
-        <v>J84</v>
+        <f t="array" aca="1" ref="F84" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L84),"$"))</f>
+        <v>L84</v>
       </c>
       <c r="G84">
         <v>4</v>
       </c>
-      <c r="I84" s="18" t="s">
-        <v>95</v>
-      </c>
-      <c r="J84" s="14" t="s">
+      <c r="K84" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="L84" s="13" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C85" t="s">
         <v>58</v>
       </c>
-      <c r="I85" s="6"/>
-      <c r="J85" s="14"/>
-    </row>
-    <row r="86" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="K85" s="5"/>
+      <c r="L85" s="13"/>
+    </row>
+    <row r="86" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B86" t="s">
         <v>79</v>
@@ -2624,29 +3086,29 @@
         <v>57</v>
       </c>
       <c r="F86" t="str" cm="1">
-        <f t="array" aca="1" ref="F86" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J86),"$"))</f>
-        <v>J86</v>
+        <f t="array" aca="1" ref="F86" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L86),"$"))</f>
+        <v>L86</v>
       </c>
       <c r="G86">
         <v>4</v>
       </c>
-      <c r="I86" s="17" t="s">
-        <v>96</v>
-      </c>
-      <c r="J86" s="13" t="s">
+      <c r="K86" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="L86" s="14" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C87" t="s">
         <v>58</v>
       </c>
-      <c r="I87" s="5"/>
-      <c r="J87" s="13"/>
-    </row>
-    <row r="88" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="K87" s="6"/>
+      <c r="L87" s="14"/>
+    </row>
+    <row r="88" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B88" t="s">
         <v>79</v>
@@ -2655,29 +3117,29 @@
         <v>57</v>
       </c>
       <c r="F88" t="str" cm="1">
-        <f t="array" aca="1" ref="F88" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J88),"$"))</f>
-        <v>J88</v>
+        <f t="array" aca="1" ref="F88" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L88),"$"))</f>
+        <v>L88</v>
       </c>
       <c r="G88">
         <v>4</v>
       </c>
-      <c r="I88" s="18" t="s">
-        <v>97</v>
-      </c>
-      <c r="J88" s="14" t="s">
+      <c r="K88" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="L88" s="13" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C89" t="s">
         <v>58</v>
       </c>
-      <c r="I89" s="6"/>
-      <c r="J89" s="14"/>
-    </row>
-    <row r="90" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="K89" s="5"/>
+      <c r="L89" s="13"/>
+    </row>
+    <row r="90" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B90" t="s">
         <v>79</v>
@@ -2686,29 +3148,29 @@
         <v>57</v>
       </c>
       <c r="F90" t="str" cm="1">
-        <f t="array" aca="1" ref="F90" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J90),"$"))</f>
-        <v>J90</v>
+        <f t="array" aca="1" ref="F90" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L90),"$"))</f>
+        <v>L90</v>
       </c>
       <c r="G90">
         <v>4</v>
       </c>
-      <c r="I90" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="J90" s="13" t="s">
+      <c r="K90" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="L90" s="14" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C91" t="s">
         <v>58</v>
       </c>
-      <c r="I91" s="5"/>
-      <c r="J91" s="13"/>
-    </row>
-    <row r="92" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="K91" s="6"/>
+      <c r="L91" s="14"/>
+    </row>
+    <row r="92" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B92" t="s">
         <v>79</v>
@@ -2717,376 +3179,407 @@
         <v>57</v>
       </c>
       <c r="F92" t="str" cm="1">
-        <f t="array" aca="1" ref="F92" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J92),"$"))</f>
-        <v>J92</v>
+        <f t="array" aca="1" ref="F92" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L92),"$"))</f>
+        <v>L92</v>
       </c>
       <c r="G92">
         <v>4</v>
       </c>
-      <c r="I92" s="18" t="s">
-        <v>102</v>
-      </c>
-      <c r="J92" s="14" t="s">
+      <c r="K92" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="L92" s="13" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C93" t="s">
         <v>58</v>
       </c>
-      <c r="I93" s="6"/>
-      <c r="J93" s="14"/>
-    </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K93" s="5"/>
+      <c r="L93" s="13"/>
+    </row>
+    <row r="94" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>93</v>
+      </c>
+      <c r="B94" t="s">
+        <v>79</v>
+      </c>
       <c r="C94" t="s">
+        <v>57</v>
+      </c>
+      <c r="F94" t="str" cm="1">
+        <f t="array" aca="1" ref="F94" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L94),"$"))</f>
+        <v>L94</v>
+      </c>
+      <c r="G94">
+        <v>4</v>
+      </c>
+      <c r="K94" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="L94" s="14" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C95" t="s">
+        <v>58</v>
+      </c>
+      <c r="K95" s="6"/>
+      <c r="L95" s="14"/>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C96" t="s">
         <v>85</v>
       </c>
-      <c r="I94" s="6"/>
-      <c r="J94" s="14"/>
-    </row>
-    <row r="95" spans="1:10" ht="75" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
+      <c r="K96" s="6"/>
+      <c r="L96" s="14"/>
+    </row>
+    <row r="97" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
         <v>104</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B97" t="s">
         <v>79</v>
       </c>
-      <c r="C95" t="s">
+      <c r="C97" t="s">
         <v>57</v>
       </c>
-      <c r="F95" t="str" cm="1">
-        <f t="array" aca="1" ref="F95" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J95),"$"))</f>
-        <v>J95</v>
-      </c>
-      <c r="G95">
-        <v>4</v>
-      </c>
-      <c r="I95" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="J95" s="13" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C96" t="s">
-        <v>58</v>
-      </c>
-      <c r="I96" s="5"/>
-      <c r="J96" s="13"/>
-    </row>
-    <row r="97" spans="1:10" ht="75" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>105</v>
-      </c>
-      <c r="B97" t="s">
-        <v>78</v>
-      </c>
       <c r="F97" t="str" cm="1">
-        <f t="array" aca="1" ref="F97" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J97),"$"))</f>
-        <v>J97</v>
+        <f t="array" aca="1" ref="F97" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L97),"$"))</f>
+        <v>L97</v>
       </c>
       <c r="G97">
         <v>4</v>
       </c>
-      <c r="I97" s="18" t="s">
+      <c r="K97" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="L97" s="13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="98" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C98" t="s">
+        <v>58</v>
+      </c>
+      <c r="K98" s="5"/>
+      <c r="L98" s="13"/>
+    </row>
+    <row r="99" spans="1:12" ht="72" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>105</v>
+      </c>
+      <c r="B99" t="s">
+        <v>78</v>
+      </c>
+      <c r="F99" t="str" cm="1">
+        <f t="array" aca="1" ref="F99" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L99),"$"))</f>
+        <v>L99</v>
+      </c>
+      <c r="G99">
+        <v>4</v>
+      </c>
+      <c r="K99" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="J97" s="14"/>
-    </row>
-    <row r="98" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
+      <c r="L99" s="14"/>
+    </row>
+    <row r="100" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
         <v>99</v>
-      </c>
-      <c r="C98" t="s">
-        <v>57</v>
-      </c>
-      <c r="F98" t="str" cm="1">
-        <f t="array" aca="1" ref="F98" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J98),"$"))</f>
-        <v>J98</v>
-      </c>
-      <c r="G98">
-        <v>4</v>
-      </c>
-      <c r="I98" s="17" t="s">
-        <v>107</v>
-      </c>
-      <c r="J98" s="13"/>
-    </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C99" t="s">
-        <v>58</v>
-      </c>
-      <c r="I99" s="5"/>
-      <c r="J99" s="13"/>
-    </row>
-    <row r="100" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>100</v>
       </c>
       <c r="C100" t="s">
         <v>57</v>
       </c>
       <c r="F100" t="str" cm="1">
-        <f t="array" aca="1" ref="F100" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J100),"$"))</f>
-        <v>J100</v>
+        <f t="array" aca="1" ref="F100" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L100),"$"))</f>
+        <v>L100</v>
       </c>
       <c r="G100">
         <v>4</v>
       </c>
-      <c r="I100" s="18" t="s">
-        <v>108</v>
-      </c>
-      <c r="J100" s="14"/>
-    </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K100" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="L100" s="13"/>
+    </row>
+    <row r="101" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C101" t="s">
         <v>58</v>
       </c>
-      <c r="I101" s="6"/>
-      <c r="J101" s="14"/>
-    </row>
-    <row r="102" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K101" s="5"/>
+      <c r="L101" s="13"/>
+    </row>
+    <row r="102" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C102" t="s">
         <v>57</v>
       </c>
       <c r="F102" t="str" cm="1">
-        <f t="array" aca="1" ref="F102" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J102),"$"))</f>
-        <v>J102</v>
+        <f t="array" aca="1" ref="F102" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L102),"$"))</f>
+        <v>L102</v>
       </c>
       <c r="G102">
         <v>4</v>
       </c>
-      <c r="I102" s="17" t="s">
-        <v>109</v>
-      </c>
-      <c r="J102" s="13"/>
-    </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K102" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="L102" s="14"/>
+    </row>
+    <row r="103" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C103" t="s">
         <v>58</v>
       </c>
-      <c r="I103" s="5"/>
-      <c r="J103" s="13"/>
-    </row>
-    <row r="104" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="K103" s="6"/>
+      <c r="L103" s="14"/>
+    </row>
+    <row r="104" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="C104" t="s">
         <v>57</v>
       </c>
       <c r="F104" t="str" cm="1">
-        <f t="array" aca="1" ref="F104" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J104),"$"))</f>
-        <v>J104</v>
+        <f t="array" aca="1" ref="F104" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L104),"$"))</f>
+        <v>L104</v>
       </c>
       <c r="G104">
-        <v>5</v>
-      </c>
-      <c r="I104" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="J104" s="14"/>
-    </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+      <c r="K104" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="L104" s="13"/>
+    </row>
+    <row r="105" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C105" t="s">
         <v>58</v>
       </c>
-      <c r="I105" s="6"/>
-      <c r="J105" s="14"/>
-    </row>
-    <row r="106" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="K105" s="5"/>
+      <c r="L105" s="13"/>
+    </row>
+    <row r="106" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C106" t="s">
         <v>57</v>
       </c>
       <c r="F106" t="str" cm="1">
-        <f t="array" aca="1" ref="F106" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",J106),"$"))</f>
-        <v>J106</v>
+        <f t="array" aca="1" ref="F106" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L106),"$"))</f>
+        <v>L106</v>
       </c>
       <c r="G106">
         <v>5</v>
       </c>
-      <c r="I106" s="17" t="s">
-        <v>115</v>
-      </c>
-      <c r="J106" s="13"/>
-    </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K106" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="L106" s="14"/>
+    </row>
+    <row r="107" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C107" t="s">
         <v>58</v>
       </c>
-      <c r="I107" s="5"/>
-      <c r="J107" s="13"/>
-    </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K107" s="6"/>
+      <c r="L107" s="14"/>
+    </row>
+    <row r="108" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>111</v>
+      </c>
       <c r="C108" t="s">
+        <v>57</v>
+      </c>
+      <c r="F108" t="str" cm="1">
+        <f t="array" aca="1" ref="F108" ca="1">_xlfn.CONCAT(_xlfn.TEXTSPLIT(CELL("address",L108),"$"))</f>
+        <v>L108</v>
+      </c>
+      <c r="G108">
+        <v>5</v>
+      </c>
+      <c r="K108" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="L108" s="13"/>
+    </row>
+    <row r="109" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C109" t="s">
+        <v>58</v>
+      </c>
+      <c r="K109" s="5"/>
+      <c r="L109" s="13"/>
+    </row>
+    <row r="110" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C110" t="s">
         <v>85</v>
       </c>
-      <c r="I108" s="5"/>
-      <c r="J108" s="13"/>
-    </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
+      <c r="K110" s="5"/>
+      <c r="L110" s="13"/>
+    </row>
+    <row r="111" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A111" t="s">
         <v>112</v>
       </c>
-      <c r="I109" s="6"/>
-      <c r="J109" s="14"/>
-    </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I110" s="5"/>
-      <c r="J110" s="13"/>
-    </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
+      <c r="K111" s="6"/>
+      <c r="L111" s="14"/>
+    </row>
+    <row r="112" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K112" s="5"/>
+      <c r="L112" s="13"/>
+    </row>
+    <row r="113" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
         <v>113</v>
       </c>
-      <c r="I111" s="6"/>
-      <c r="J111" s="14"/>
-    </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I112" s="5"/>
-      <c r="J112" s="13"/>
-    </row>
-    <row r="113" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I113" s="6"/>
-      <c r="J113" s="14"/>
-    </row>
-    <row r="114" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I114" s="5"/>
-      <c r="J114" s="13"/>
-    </row>
-    <row r="115" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I115" s="6"/>
-      <c r="J115" s="14"/>
-    </row>
-    <row r="116" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I116" s="5"/>
-      <c r="J116" s="13"/>
-    </row>
-    <row r="117" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I117" s="6"/>
-      <c r="J117" s="14"/>
-    </row>
-    <row r="118" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I118" s="20" t="s">
+      <c r="K113" s="6"/>
+      <c r="L113" s="14"/>
+    </row>
+    <row r="114" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K114" s="5"/>
+      <c r="L114" s="13"/>
+    </row>
+    <row r="115" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K115" s="6"/>
+      <c r="L115" s="14"/>
+    </row>
+    <row r="116" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K116" s="5"/>
+      <c r="L116" s="13"/>
+    </row>
+    <row r="117" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K117" s="6"/>
+      <c r="L117" s="14"/>
+    </row>
+    <row r="118" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K118" s="5"/>
+      <c r="L118" s="13"/>
+    </row>
+    <row r="119" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K119" s="6"/>
+      <c r="L119" s="14"/>
+    </row>
+    <row r="120" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K120" s="18" t="s">
         <v>116</v>
       </c>
-      <c r="J118" s="20"/>
+      <c r="L120" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="I76:J76"/>
-    <mergeCell ref="I118:J118"/>
-    <mergeCell ref="I47:J47"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="K78:L78"/>
+    <mergeCell ref="K120:L120"/>
+    <mergeCell ref="K49:L49"/>
+    <mergeCell ref="K36:L36"/>
+    <mergeCell ref="K41:L41"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="K20:L20"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
-  <conditionalFormatting sqref="C7 C9 C11 C13 C15 C17 C19 C21 C23 C25 C27 C29 C31 C33 C35 C37 C39 C41 C43 C45 C47 C49 C51 C53 C55 C57 C59 C67 C69 C71 C73 C75">
-    <cfRule type="expression" dxfId="8" priority="12">
-      <formula>ISBLANK(C7)</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="C3 C5">
     <cfRule type="expression" dxfId="7" priority="1">
       <formula>ISBLANK(C3)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C8 C10 C12 C14 C16 C18 C20 C22 C24 C26 C28 C30 C32 C34 C36 C38 C40 C42 C44 C46 C48 C50 C52 C54 C56 C58 C60 C66 C68 C70 C72 C74 C76:C77">
-    <cfRule type="expression" dxfId="6" priority="7">
+  <conditionalFormatting sqref="C7 C9 C11 C13 C15 C17 C19 C21:C22 C25 C27 C29 C31 C33 C35 C37 C39 C41 C43 C45 C47 C49 C51 C53 C55 C57 C59 C61 C69 C71 C73 C75 C77">
+    <cfRule type="expression" dxfId="6" priority="12">
+      <formula>ISBLANK(C7)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C8 C10 C12 C14 C16 C18 C20 C23:C24 C26 C28 C30 C32 C34 C36 C38 C40 C42 C44 C46 C48 C50 C52 C54 C56 C58 C60 C62 C68 C70 C72 C74 C76 C78:C79">
+    <cfRule type="expression" dxfId="5" priority="7">
       <formula>ISBLANK(C8)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C78:C79">
-    <cfRule type="expression" dxfId="5" priority="4">
-      <formula>ISBLANK(C78)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C80">
-    <cfRule type="expression" dxfId="4" priority="3">
+  <conditionalFormatting sqref="C80:C81">
+    <cfRule type="expression" dxfId="4" priority="4">
       <formula>ISBLANK(C80)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C81">
-    <cfRule type="expression" dxfId="3" priority="2">
-      <formula>ISBLANK(C81)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C82 C84 C86 C88 C90 C92 C94 C96:C97 C99 C101 C103 C105 C107 C109 C111 C113 C115 C117">
-    <cfRule type="expression" dxfId="2" priority="5">
+  <conditionalFormatting sqref="C82">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>ISBLANK(C82)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C83 C85 C87 C89 C91 C93 C95 C98 C100 C102 C104 C106 C108 C110 C112 C114 C116">
-    <cfRule type="expression" dxfId="1" priority="6">
+  <conditionalFormatting sqref="C83">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>ISBLANK(C83)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C84 C86 C88 C90 C92 C94 C96 C98:C99 C101 C103 C105 C107 C109 C111 C113 C115 C117 C119">
+    <cfRule type="expression" dxfId="1" priority="5">
+      <formula>ISBLANK(C84)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C85 C87 C89 C91 C93 C95 C97 C100 C102 C104 C106 C108 C110 C112 C114 C116 C118">
+    <cfRule type="expression" dxfId="0" priority="6">
+      <formula>ISBLANK(C85)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="16">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2" xr:uid="{DBDA0B2E-73C7-461D-9A78-8C9C0FC3C8EE}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2" xr:uid="{DBDA0B2E-73C7-461D-9A78-8C9C0FC3C8EE}">
       <formula1>$C$2:$C$6</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J27" xr:uid="{2A4FBB3A-AF25-40CF-A7C5-68C363A144AC}">
-      <formula1>$F$27:$F$31</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L29" xr:uid="{2A4FBB3A-AF25-40CF-A7C5-68C363A144AC}">
+      <formula1>$F$29:$F$33</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J32" xr:uid="{4F3AB38D-0522-46BE-8207-6886168C0716}">
-      <formula1>$F$32:$F$33</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L34" xr:uid="{4F3AB38D-0522-46BE-8207-6886168C0716}">
+      <formula1>$F$34:$F$35</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J41" xr:uid="{C7C9BACE-9E87-4F51-B7AA-AF028398DF42}">
-      <formula1>$C$41:$C$42</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L43" xr:uid="{C7C9BACE-9E87-4F51-B7AA-AF028398DF42}">
+      <formula1>$C$43:$C$44</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J59" xr:uid="{3E2DD406-56CF-445C-BD6B-86CB8C7B00BA}">
-      <formula1>$C$59:$C$60</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L61" xr:uid="{3E2DD406-56CF-445C-BD6B-86CB8C7B00BA}">
+      <formula1>$C$61:$C$62</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J66" xr:uid="{2281ACFD-B768-49F6-AC73-6654DDA39B30}">
-      <formula1>$C$66:$C$67</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L68" xr:uid="{2281ACFD-B768-49F6-AC73-6654DDA39B30}">
+      <formula1>$C$68:$C$69</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J61" xr:uid="{8C1D64B0-BEF7-4B52-B632-2C0C338A42F7}">
-      <formula1>$C$61:$C$65</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L63" xr:uid="{8C1D64B0-BEF7-4B52-B632-2C0C338A42F7}">
+      <formula1>$C$63:$C$67</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J77" xr:uid="{6C1903ED-8B8C-48BC-919C-F2058E6A8659}">
-      <formula1>$C$77:$C$79</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L79" xr:uid="{6C1903ED-8B8C-48BC-919C-F2058E6A8659}">
+      <formula1>$C$79:$C$81</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J80" xr:uid="{ACFB3B64-C620-4E47-92D2-33CF0053623A}">
-      <formula1>$C$80:$C$81</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J82" xr:uid="{5EDB7A92-9ABD-414D-853E-147436B3DF5B}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L82" xr:uid="{ACFB3B64-C620-4E47-92D2-33CF0053623A}">
       <formula1>$C$82:$C$83</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J84" xr:uid="{F4A03EBA-03ED-4032-A0D1-343727C4795F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L84" xr:uid="{5EDB7A92-9ABD-414D-853E-147436B3DF5B}">
       <formula1>$C$84:$C$85</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J86" xr:uid="{E8E2CD95-F50E-4FF7-ABC6-86296DBBA686}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L86" xr:uid="{F4A03EBA-03ED-4032-A0D1-343727C4795F}">
       <formula1>$C$86:$C$87</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J88" xr:uid="{0B1BA240-F98F-432F-848E-5BB4A2491089}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L88" xr:uid="{E8E2CD95-F50E-4FF7-ABC6-86296DBBA686}">
       <formula1>$C$88:$C$89</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J90" xr:uid="{BA661406-18B5-499D-805E-2915FA9F0DF9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L90" xr:uid="{0B1BA240-F98F-432F-848E-5BB4A2491089}">
       <formula1>$C$90:$C$91</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J92" xr:uid="{9F5640E1-D879-422F-A55D-D83374471FF5}">
-      <formula1>$C$92:$C$94</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L92" xr:uid="{BA661406-18B5-499D-805E-2915FA9F0DF9}">
+      <formula1>$C$92:$C$93</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J95" xr:uid="{2BC6887D-D646-42E9-A274-3D9790A1E66B}">
-      <formula1>$C$95:$C$96</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L94" xr:uid="{9F5640E1-D879-422F-A55D-D83374471FF5}">
+      <formula1>$C$94:$C$96</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L97" xr:uid="{2BC6887D-D646-42E9-A274-3D9790A1E66B}">
+      <formula1>$C$97:$C$98</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="J19" r:id="rId1" xr:uid="{F23C4D8F-D3A5-41F8-8768-957B6ED66387}"/>
-    <hyperlink ref="J38" r:id="rId2" xr:uid="{7C1EE75F-8A56-4E1F-8F6D-E3D927261E7F}"/>
-    <hyperlink ref="J45" r:id="rId3" display="random@icould.com" xr:uid="{0D1B7BBF-15B3-4CFC-9039-2B5392E32994}"/>
+    <hyperlink ref="L19" r:id="rId1" xr:uid="{F23C4D8F-D3A5-41F8-8768-957B6ED66387}"/>
+    <hyperlink ref="L40" r:id="rId2" xr:uid="{7C1EE75F-8A56-4E1F-8F6D-E3D927261E7F}"/>
+    <hyperlink ref="L47" r:id="rId3" display="random@icould.com" xr:uid="{0D1B7BBF-15B3-4CFC-9039-2B5392E32994}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId4"/>
@@ -3097,43 +3590,43 @@
           <x14:formula1>
             <xm:f>Backend!$B$2:$B$6</xm:f>
           </x14:formula1>
-          <xm:sqref>J28:J31</xm:sqref>
+          <xm:sqref>L30:L33</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B3132453-0252-43A7-BEC0-13862065EF0E}">
           <x14:formula1>
             <xm:f>Backend!$C$2:$C$3</xm:f>
           </x14:formula1>
-          <xm:sqref>J33</xm:sqref>
+          <xm:sqref>L35</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{30E8FBE2-C2FC-4B6D-9F98-1AD125B8C425}">
           <x14:formula1>
             <xm:f>Backend!$E$2:$E$3</xm:f>
           </x14:formula1>
-          <xm:sqref>J42</xm:sqref>
+          <xm:sqref>L44</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D7F0EB7B-BBFF-45D3-B222-8DBEA2A4E2AA}">
           <x14:formula1>
             <xm:f>Backend!$F$2:$F$3</xm:f>
           </x14:formula1>
-          <xm:sqref>J60 J67</xm:sqref>
+          <xm:sqref>L62 L69</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{85EB1F5D-2C0D-4619-81F3-F49B63FA8937}">
           <x14:formula1>
             <xm:f>Backend!$G$2:$G$6</xm:f>
           </x14:formula1>
-          <xm:sqref>J62:J65</xm:sqref>
+          <xm:sqref>L64:L67</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3BF7E381-8828-457B-A727-E2C5CC93B0AF}">
           <x14:formula1>
             <xm:f>Backend!$H$2:$H$6</xm:f>
           </x14:formula1>
-          <xm:sqref>J71:J75</xm:sqref>
+          <xm:sqref>L73:L77</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F3641AE7-F3E1-4130-BA9D-61DF5A2A44B2}">
           <x14:formula1>
             <xm:f>Backend!$I$2:$I$3</xm:f>
           </x14:formula1>
-          <xm:sqref>B97 B76:B77 B80 B82 B84 B86 B88 B90 B92 B95 B2:B71</xm:sqref>
+          <xm:sqref>B99 B78:B79 B82 B84 B86 B88 B90 B92 B94 B97 B2:B73</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3145,19 +3638,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC180A74-45BA-42EE-9251-9C730233F3C6}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:I1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.140625" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.109375" customWidth="1"/>
     <col min="8" max="8" width="18" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>

</xml_diff>